<commit_message>
updated cost template with instructions
</commit_message>
<xml_diff>
--- a/www/cost-template-empty_Francais.xlsx
+++ b/www/cost-template-empty_Francais.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hthompson\OneDrive - PATH\Documents\github\malaria-budgeting-tool\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{092CDCBE-ACEB-4FA6-A4FA-85723A6DD715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF9FDC7F-223B-44C5-8505-A132FABD403E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{E72D83C0-31FE-469B-BB4E-361133B71EB0}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="119">
   <si>
     <t>code_intervention</t>
   </si>
@@ -333,6 +333,619 @@
   </si>
   <si>
     <t>facteur_d'inflation_initial_à_l'annee_d'analyse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assurez-vous que les en-têtes de colonne des colonnes A : J restent inchangés et que des colonnes supplémentaires peuvent être ajoutées selon les besoins de l'utilisateur. </t>
+  </si>
+  <si>
+    <t>Des feuilles supplémentaires pour le suivi des calculs de coûts unitaires, par exemple, peuvent également être ajoutées librement.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les cellules ne contiennent pas de formules prédéfinies et c'est à l'utilisateur de saisir ou de calculer les données comme il l'entend.  </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Le modèle est prérempli avec certaines interventions, types d'intervention, classes de coûts et unités courants – ces lignes peuvent être modifiées et/ou supprimées selon les besoins de l'utilisateur, mais assurez-vous que pour chaque intervention réalisée dans le </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>plan opérationnel</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>, il y a des coûts unitaires pour l'intervention spécifique et le type d'intervention.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">S'il le souhaite, l'utilisateur peut également ajouter des coûts unitaires spécifiques à l'emplacement. Pour ce faire, ajoutez des colonnes supplémentaires pour les spécifications 'adm1' et adm2' et assurez-vous que les noms sont cohérents entre celle-ci et la feuille de calcul du mix d'intervention, l'outil s'occupera du reste! </t>
+  </si>
+  <si>
+    <t>Remplissez le modèle Excel :</t>
+  </si>
+  <si>
+    <r>
+      <t>·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">         </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>'</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">code_intervention' : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Sélectionnez dans la liste déroulante l'intervention à laquelle les données de coût se rapportent. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">         </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">type_intervention : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Sélectionnez dans la liste déroulante le type d'intervention spécifique auquel le coût se rapporte. Ces valeurs se rapportent à la colonne «</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> type_ » </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">du modèle précédent. Si l'utilisateur souhaite inclure des coûts fixes pour une intervention, cela est également spécifié dans cette colonne, par exemple Coûts fixes pour l'entreposage annuel de moustiquaires au cours d'une campagne. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">         </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">cout_classe : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Sélectionnez la classe de coûts (</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Approvisionnement, Distribution, Opérationnel, Support, Autre</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) Si vous sélectionnez «</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> autre »,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> indiquez dans la colonne</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> « cout_classe_autre » </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">de quoi il s'agit. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">         </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">'description' : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>fournissez une brève description des composants du coût unitaire dans la colonne de description.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">         </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">'unite' : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Sélectionnez dans la liste déroulante l'unité spécifique pour le coût, par exemple </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">par filet, par enfant, par dose, par an </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, etc  </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">         </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>'cout_monnaie_locale'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> : Valeur monétaire du coût unitaire spécifique en CDF </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">         </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">'taux_de_change' : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">taux de change à convertir de CDF en USD pour renseigner les valeurs de coût unitaire dans la </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> colonne 'cout_usd</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">.  </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">         </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">'count_annee_pour_analyse' : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">cette valeur est l'année du plan opérationnel pour lequel le coût unitaire doit être utilisé pour calculer le budget. Si cette colonne est laissée vide, le même coût unitaire sera appliqué pour chaque année de livraison dans le plan spécifié. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">         </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Pour faciliter la conversion des estimations de coût unitaire générées à partir de données historiques en valeurs monétaires actuelles, il existe les colonnes supplémentaires suivantes pour faciliter cette tâche : </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">cout_unitaire_d'origine l' </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">estimation du coût unitaire d'origine, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">cout_unitaire_original_annee </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">l'année des données utilisées pour estimer le coût unitaire et enfin </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">'facteur_d'inflation_initial_à_l'année_d'analyse' </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">le facteur d'inflation à appliquer pour avoir des coûts unitaires en valeurs attendues actuelles et futures. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">         </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Les colonnes 'Notes' </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">et </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">'Source' </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">peuvent être utilisées pour stocker des notes et des détails spécifiques sur la source de données utilisée pour générer les coûts unitaires. </t>
+    </r>
+  </si>
+  <si>
+    <t>Une fois que les données de coût unitaire ont été spécifiées, l'utilisateur peut enregistrer une copie locale de ce fichier.</t>
+  </si>
+  <si>
+    <r>
+      <t>Revenez à l'application Web et téléchargez le fichier Excel complété à l'aide du formulaire et donnez à la feuille de coûts un nom : par exemple «</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Coût 1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">», etc. et une description : par exemple « </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Basé sur les données de coûts historiques </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>» – assurez-vous qu'il s'agit de descriptions informatives car elles seront utiles lors de la génération et de la comparaison des plans.</t>
+    </r>
+  </si>
+  <si>
+    <t>Appuyez sur le bouton « Soumettre la feuille de coûts » et la feuille de calcul sera téléchargée dans l'outil.</t>
+  </si>
+  <si>
+    <t>Les données de coût téléchargées apparaîtront dans un tableau récapitulatif.</t>
+  </si>
+  <si>
+    <t>Comment utiliser</t>
   </si>
 </sst>
 </file>
@@ -343,7 +956,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -482,6 +1095,46 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Symbol"/>
+      <family val="1"/>
+      <charset val="2"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="22"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="35">
@@ -842,14 +1495,30 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
     </xf>
   </cellXfs>
   <cellStyles count="47">
@@ -915,6 +1584,55 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>142875</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>104775</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>188461</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Une capture d'écran d'un ordinateur&#10;&#10;Le contenu généré par l'IA peut être incorrect.">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0E3B4705-0E57-4910-995D-4063E4B00867}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1362075" y="5391150"/>
+          <a:ext cx="11544300" cy="5541511"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
@@ -1296,254 +2014,1866 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{649389F8-E97B-47EA-A957-AF7402F6F82B}">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:W73"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="2"/>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
+    <row r="1" spans="1:23" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+      <c r="Q1" s="4"/>
+      <c r="R1" s="4"/>
+      <c r="S1" s="4"/>
+      <c r="T1" s="4"/>
+      <c r="U1" s="4"/>
+      <c r="V1" s="4"/>
+      <c r="W1" s="4"/>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+      <c r="P2" s="5"/>
+      <c r="Q2" s="5"/>
+      <c r="R2" s="5"/>
+      <c r="S2" s="5"/>
+      <c r="T2" s="5"/>
+      <c r="U2" s="5"/>
+      <c r="V2" s="5"/>
+      <c r="W2" s="5"/>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
+      <c r="R3" s="5"/>
+      <c r="S3" s="5"/>
+      <c r="T3" s="5"/>
+      <c r="U3" s="5"/>
+      <c r="V3" s="5"/>
+      <c r="W3" s="5"/>
+    </row>
+    <row r="4" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="5"/>
+      <c r="O4" s="5"/>
+      <c r="P4" s="5"/>
+      <c r="Q4" s="5"/>
+      <c r="R4" s="5"/>
+      <c r="S4" s="5"/>
+      <c r="T4" s="5"/>
+      <c r="U4" s="5"/>
+      <c r="V4" s="5"/>
+      <c r="W4" s="5"/>
+    </row>
+    <row r="5" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="5"/>
+      <c r="N5" s="5"/>
+      <c r="O5" s="5"/>
+      <c r="P5" s="5"/>
+      <c r="Q5" s="5"/>
+      <c r="R5" s="5"/>
+      <c r="S5" s="5"/>
+      <c r="T5" s="5"/>
+      <c r="U5" s="5"/>
+      <c r="V5" s="5"/>
+      <c r="W5" s="5"/>
+    </row>
+    <row r="6" spans="1:23" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="5"/>
+      <c r="N6" s="5"/>
+      <c r="O6" s="5"/>
+      <c r="P6" s="5"/>
+      <c r="Q6" s="5"/>
+      <c r="R6" s="5"/>
+      <c r="S6" s="5"/>
+      <c r="T6" s="5"/>
+      <c r="U6" s="5"/>
+      <c r="V6" s="5"/>
+      <c r="W6" s="5"/>
+    </row>
+    <row r="7" spans="1:23" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="8"/>
+      <c r="R7" s="8"/>
+      <c r="S7" s="8"/>
+      <c r="T7" s="8"/>
+      <c r="U7" s="8"/>
+      <c r="V7" s="8"/>
+      <c r="W7" s="5"/>
+    </row>
+    <row r="8" spans="1:23" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="8"/>
+      <c r="S8" s="8"/>
+      <c r="T8" s="8"/>
+      <c r="U8" s="8"/>
+      <c r="V8" s="8"/>
+      <c r="W8" s="5"/>
+    </row>
+    <row r="9" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
+      <c r="O9" s="5"/>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="5"/>
+      <c r="S9" s="5"/>
+      <c r="T9" s="5"/>
+      <c r="U9" s="5"/>
+      <c r="V9" s="5"/>
+      <c r="W9" s="5"/>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="5"/>
+      <c r="P10" s="5"/>
+      <c r="Q10" s="5"/>
+      <c r="R10" s="5"/>
+      <c r="S10" s="5"/>
+      <c r="T10" s="5"/>
+      <c r="U10" s="5"/>
+      <c r="V10" s="5"/>
+      <c r="W10" s="5"/>
+    </row>
+    <row r="11" spans="1:23" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="9"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="9"/>
+      <c r="O11" s="9"/>
+      <c r="P11" s="9"/>
+      <c r="Q11" s="9"/>
+      <c r="R11" s="9"/>
+      <c r="S11" s="9"/>
+      <c r="T11" s="9"/>
+      <c r="U11" s="9"/>
+      <c r="V11" s="9"/>
+      <c r="W11" s="5"/>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="5"/>
+      <c r="L12" s="5"/>
+      <c r="M12" s="5"/>
+      <c r="N12" s="5"/>
+      <c r="O12" s="5"/>
+      <c r="P12" s="5"/>
+      <c r="Q12" s="5"/>
+      <c r="R12" s="5"/>
+      <c r="S12" s="5"/>
+      <c r="T12" s="5"/>
+      <c r="U12" s="5"/>
+      <c r="V12" s="5"/>
+      <c r="W12" s="5"/>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
+      <c r="N13" s="5"/>
+      <c r="O13" s="5"/>
+      <c r="P13" s="5"/>
+      <c r="Q13" s="5"/>
+      <c r="R13" s="5"/>
+      <c r="S13" s="5"/>
+      <c r="T13" s="5"/>
+      <c r="U13" s="5"/>
+      <c r="V13" s="5"/>
+      <c r="W13" s="5"/>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="5"/>
+      <c r="O14" s="5"/>
+      <c r="P14" s="5"/>
+      <c r="Q14" s="5"/>
+      <c r="R14" s="5"/>
+      <c r="S14" s="5"/>
+      <c r="T14" s="5"/>
+      <c r="U14" s="5"/>
+      <c r="V14" s="5"/>
+      <c r="W14" s="5"/>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
+      <c r="L15" s="5"/>
+      <c r="M15" s="5"/>
+      <c r="N15" s="5"/>
+      <c r="O15" s="5"/>
+      <c r="P15" s="5"/>
+      <c r="Q15" s="5"/>
+      <c r="R15" s="5"/>
+      <c r="S15" s="5"/>
+      <c r="T15" s="5"/>
+      <c r="U15" s="5"/>
+      <c r="V15" s="5"/>
+      <c r="W15" s="5"/>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+      <c r="L16" s="5"/>
+      <c r="M16" s="5"/>
+      <c r="N16" s="5"/>
+      <c r="O16" s="5"/>
+      <c r="P16" s="5"/>
+      <c r="Q16" s="5"/>
+      <c r="R16" s="5"/>
+      <c r="S16" s="5"/>
+      <c r="T16" s="5"/>
+      <c r="U16" s="5"/>
+      <c r="V16" s="5"/>
+      <c r="W16" s="5"/>
+    </row>
+    <row r="17" spans="1:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="9"/>
+      <c r="K17" s="9"/>
+      <c r="L17" s="9"/>
+      <c r="M17" s="9"/>
+      <c r="N17" s="9"/>
+      <c r="O17" s="9"/>
+      <c r="P17" s="9"/>
+      <c r="Q17" s="9"/>
+      <c r="R17" s="9"/>
+      <c r="S17" s="9"/>
+      <c r="T17" s="9"/>
+      <c r="U17" s="9"/>
+      <c r="V17" s="9"/>
+      <c r="W17" s="9"/>
+    </row>
+    <row r="18" spans="1:23" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="9"/>
+      <c r="K18" s="9"/>
+      <c r="L18" s="9"/>
+      <c r="M18" s="9"/>
+      <c r="N18" s="9"/>
+      <c r="O18" s="9"/>
+      <c r="P18" s="9"/>
+      <c r="Q18" s="9"/>
+      <c r="R18" s="9"/>
+      <c r="S18" s="9"/>
+      <c r="T18" s="9"/>
+      <c r="U18" s="9"/>
+      <c r="V18" s="9"/>
+      <c r="W18" s="9"/>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="5"/>
+      <c r="L19" s="5"/>
+      <c r="M19" s="5"/>
+      <c r="N19" s="5"/>
+      <c r="O19" s="5"/>
+      <c r="P19" s="5"/>
+      <c r="Q19" s="5"/>
+      <c r="R19" s="5"/>
+      <c r="S19" s="5"/>
+      <c r="T19" s="5"/>
+      <c r="U19" s="5"/>
+      <c r="V19" s="5"/>
+      <c r="W19" s="5"/>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
+      <c r="N20" s="5"/>
+      <c r="O20" s="5"/>
+      <c r="P20" s="5"/>
+      <c r="Q20" s="5"/>
+      <c r="R20" s="5"/>
+      <c r="S20" s="5"/>
+      <c r="T20" s="5"/>
+      <c r="U20" s="5"/>
+      <c r="V20" s="5"/>
+      <c r="W20" s="5"/>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="5"/>
+      <c r="L21" s="5"/>
+      <c r="M21" s="5"/>
+      <c r="N21" s="5"/>
+      <c r="O21" s="5"/>
+      <c r="P21" s="5"/>
+      <c r="Q21" s="5"/>
+      <c r="R21" s="5"/>
+      <c r="S21" s="5"/>
+      <c r="T21" s="5"/>
+      <c r="U21" s="5"/>
+      <c r="V21" s="5"/>
+      <c r="W21" s="5"/>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A22" s="3"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="5"/>
+      <c r="L22" s="5"/>
+      <c r="M22" s="5"/>
+      <c r="N22" s="5"/>
+      <c r="O22" s="5"/>
+      <c r="P22" s="5"/>
+      <c r="Q22" s="5"/>
+      <c r="R22" s="5"/>
+      <c r="S22" s="5"/>
+      <c r="T22" s="5"/>
+      <c r="U22" s="5"/>
+      <c r="V22" s="5"/>
+      <c r="W22" s="5"/>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A23" s="3"/>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="5"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="5"/>
+      <c r="L23" s="5"/>
+      <c r="M23" s="5"/>
+      <c r="N23" s="5"/>
+      <c r="O23" s="5"/>
+      <c r="P23" s="5"/>
+      <c r="Q23" s="5"/>
+      <c r="R23" s="5"/>
+      <c r="S23" s="5"/>
+      <c r="T23" s="5"/>
+      <c r="U23" s="5"/>
+      <c r="V23" s="5"/>
+      <c r="W23" s="5"/>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A24" s="3"/>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="5"/>
+      <c r="J24" s="5"/>
+      <c r="K24" s="5"/>
+      <c r="L24" s="5"/>
+      <c r="M24" s="5"/>
+      <c r="N24" s="5"/>
+      <c r="O24" s="5"/>
+      <c r="P24" s="5"/>
+      <c r="Q24" s="5"/>
+      <c r="R24" s="5"/>
+      <c r="S24" s="5"/>
+      <c r="T24" s="5"/>
+      <c r="U24" s="5"/>
+      <c r="V24" s="5"/>
+      <c r="W24" s="5"/>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A25" s="5"/>
+      <c r="B25" s="5"/>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="5"/>
+      <c r="L25" s="5"/>
+      <c r="M25" s="5"/>
+      <c r="N25" s="5"/>
+      <c r="O25" s="5"/>
+      <c r="P25" s="5"/>
+      <c r="Q25" s="5"/>
+      <c r="R25" s="5"/>
+      <c r="S25" s="5"/>
+      <c r="T25" s="5"/>
+      <c r="U25" s="5"/>
+      <c r="V25" s="5"/>
+      <c r="W25" s="5"/>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A26" s="5"/>
+      <c r="B26" s="5"/>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+      <c r="I26" s="5"/>
+      <c r="J26" s="5"/>
+      <c r="K26" s="5"/>
+      <c r="L26" s="5"/>
+      <c r="M26" s="5"/>
+      <c r="N26" s="5"/>
+      <c r="O26" s="5"/>
+      <c r="P26" s="5"/>
+      <c r="Q26" s="5"/>
+      <c r="R26" s="5"/>
+      <c r="S26" s="5"/>
+      <c r="T26" s="5"/>
+      <c r="U26" s="5"/>
+      <c r="V26" s="5"/>
+      <c r="W26" s="5"/>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A27" s="5"/>
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+      <c r="I27" s="5"/>
+      <c r="J27" s="5"/>
+      <c r="K27" s="5"/>
+      <c r="L27" s="5"/>
+      <c r="M27" s="5"/>
+      <c r="N27" s="5"/>
+      <c r="O27" s="5"/>
+      <c r="P27" s="5"/>
+      <c r="Q27" s="5"/>
+      <c r="R27" s="5"/>
+      <c r="S27" s="5"/>
+      <c r="T27" s="5"/>
+      <c r="U27" s="5"/>
+      <c r="V27" s="5"/>
+      <c r="W27" s="5"/>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A28" s="5"/>
+      <c r="B28" s="5"/>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="5"/>
+      <c r="I28" s="5"/>
+      <c r="J28" s="5"/>
+      <c r="K28" s="5"/>
+      <c r="L28" s="5"/>
+      <c r="M28" s="5"/>
+      <c r="N28" s="5"/>
+      <c r="O28" s="5"/>
+      <c r="P28" s="5"/>
+      <c r="Q28" s="5"/>
+      <c r="R28" s="5"/>
+      <c r="S28" s="5"/>
+      <c r="T28" s="5"/>
+      <c r="U28" s="5"/>
+      <c r="V28" s="5"/>
+      <c r="W28" s="5"/>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A29" s="5"/>
+      <c r="B29" s="5"/>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+      <c r="I29" s="5"/>
+      <c r="J29" s="5"/>
+      <c r="K29" s="5"/>
+      <c r="L29" s="5"/>
+      <c r="M29" s="5"/>
+      <c r="N29" s="5"/>
+      <c r="O29" s="5"/>
+      <c r="P29" s="5"/>
+      <c r="Q29" s="5"/>
+      <c r="R29" s="5"/>
+      <c r="S29" s="5"/>
+      <c r="T29" s="5"/>
+      <c r="U29" s="5"/>
+      <c r="V29" s="5"/>
+      <c r="W29" s="5"/>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A30" s="5"/>
+      <c r="B30" s="5"/>
+      <c r="C30" s="5"/>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
+      <c r="G30" s="5"/>
+      <c r="H30" s="5"/>
+      <c r="I30" s="5"/>
+      <c r="J30" s="5"/>
+      <c r="K30" s="5"/>
+      <c r="L30" s="5"/>
+      <c r="M30" s="5"/>
+      <c r="N30" s="5"/>
+      <c r="O30" s="5"/>
+      <c r="P30" s="5"/>
+      <c r="Q30" s="5"/>
+      <c r="R30" s="5"/>
+      <c r="S30" s="5"/>
+      <c r="T30" s="5"/>
+      <c r="U30" s="5"/>
+      <c r="V30" s="5"/>
+      <c r="W30" s="5"/>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A31" s="5"/>
+      <c r="B31" s="5"/>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="5"/>
+      <c r="I31" s="5"/>
+      <c r="J31" s="5"/>
+      <c r="K31" s="5"/>
+      <c r="L31" s="5"/>
+      <c r="M31" s="5"/>
+      <c r="N31" s="5"/>
+      <c r="O31" s="5"/>
+      <c r="P31" s="5"/>
+      <c r="Q31" s="5"/>
+      <c r="R31" s="5"/>
+      <c r="S31" s="5"/>
+      <c r="T31" s="5"/>
+      <c r="U31" s="5"/>
+      <c r="V31" s="5"/>
+      <c r="W31" s="5"/>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A32" s="5"/>
+      <c r="B32" s="5"/>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+      <c r="I32" s="5"/>
+      <c r="J32" s="5"/>
+      <c r="K32" s="5"/>
+      <c r="L32" s="5"/>
+      <c r="M32" s="5"/>
+      <c r="N32" s="5"/>
+      <c r="O32" s="5"/>
+      <c r="P32" s="5"/>
+      <c r="Q32" s="5"/>
+      <c r="R32" s="5"/>
+      <c r="S32" s="5"/>
+      <c r="T32" s="5"/>
+      <c r="U32" s="5"/>
+      <c r="V32" s="5"/>
+      <c r="W32" s="5"/>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A33" s="5"/>
+      <c r="B33" s="5"/>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="5"/>
+      <c r="L33" s="5"/>
+      <c r="M33" s="5"/>
+      <c r="N33" s="5"/>
+      <c r="O33" s="5"/>
+      <c r="P33" s="5"/>
+      <c r="Q33" s="5"/>
+      <c r="R33" s="5"/>
+      <c r="S33" s="5"/>
+      <c r="T33" s="5"/>
+      <c r="U33" s="5"/>
+      <c r="V33" s="5"/>
+      <c r="W33" s="5"/>
+    </row>
+    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A34" s="5"/>
+      <c r="B34" s="5"/>
+      <c r="C34" s="5"/>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="5"/>
+      <c r="I34" s="5"/>
+      <c r="J34" s="5"/>
+      <c r="K34" s="5"/>
+      <c r="L34" s="5"/>
+      <c r="M34" s="5"/>
+      <c r="N34" s="5"/>
+      <c r="O34" s="5"/>
+      <c r="P34" s="5"/>
+      <c r="Q34" s="5"/>
+      <c r="R34" s="5"/>
+      <c r="S34" s="5"/>
+      <c r="T34" s="5"/>
+      <c r="U34" s="5"/>
+      <c r="V34" s="5"/>
+      <c r="W34" s="5"/>
+    </row>
+    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A35" s="5"/>
+      <c r="B35" s="5"/>
+      <c r="C35" s="5"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5"/>
+      <c r="I35" s="5"/>
+      <c r="J35" s="5"/>
+      <c r="K35" s="5"/>
+      <c r="L35" s="5"/>
+      <c r="M35" s="5"/>
+      <c r="N35" s="5"/>
+      <c r="O35" s="5"/>
+      <c r="P35" s="5"/>
+      <c r="Q35" s="5"/>
+      <c r="R35" s="5"/>
+      <c r="S35" s="5"/>
+      <c r="T35" s="5"/>
+      <c r="U35" s="5"/>
+      <c r="V35" s="5"/>
+      <c r="W35" s="5"/>
+    </row>
+    <row r="36" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A36" s="5"/>
+      <c r="B36" s="5"/>
+      <c r="C36" s="5"/>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5"/>
+      <c r="I36" s="5"/>
+      <c r="J36" s="5"/>
+      <c r="K36" s="5"/>
+      <c r="L36" s="5"/>
+      <c r="M36" s="5"/>
+      <c r="N36" s="5"/>
+      <c r="O36" s="5"/>
+      <c r="P36" s="5"/>
+      <c r="Q36" s="5"/>
+      <c r="R36" s="5"/>
+      <c r="S36" s="5"/>
+      <c r="T36" s="5"/>
+      <c r="U36" s="5"/>
+      <c r="V36" s="5"/>
+      <c r="W36" s="5"/>
+    </row>
+    <row r="37" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A37" s="5"/>
+      <c r="B37" s="5"/>
+      <c r="C37" s="5"/>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="5"/>
+      <c r="H37" s="5"/>
+      <c r="I37" s="5"/>
+      <c r="J37" s="5"/>
+      <c r="K37" s="5"/>
+      <c r="L37" s="5"/>
+      <c r="M37" s="5"/>
+      <c r="N37" s="5"/>
+      <c r="O37" s="5"/>
+      <c r="P37" s="5"/>
+      <c r="Q37" s="5"/>
+      <c r="R37" s="5"/>
+      <c r="S37" s="5"/>
+      <c r="T37" s="5"/>
+      <c r="U37" s="5"/>
+      <c r="V37" s="5"/>
+      <c r="W37" s="5"/>
+    </row>
+    <row r="38" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A38" s="5"/>
+      <c r="B38" s="5"/>
+      <c r="C38" s="5"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="5"/>
+      <c r="G38" s="5"/>
+      <c r="H38" s="5"/>
+      <c r="I38" s="5"/>
+      <c r="J38" s="5"/>
+      <c r="K38" s="5"/>
+      <c r="L38" s="5"/>
+      <c r="M38" s="5"/>
+      <c r="N38" s="5"/>
+      <c r="O38" s="5"/>
+      <c r="P38" s="5"/>
+      <c r="Q38" s="5"/>
+      <c r="R38" s="5"/>
+      <c r="S38" s="5"/>
+      <c r="T38" s="5"/>
+      <c r="U38" s="5"/>
+      <c r="V38" s="5"/>
+      <c r="W38" s="5"/>
+    </row>
+    <row r="39" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A39" s="5"/>
+      <c r="B39" s="5"/>
+      <c r="C39" s="5"/>
+      <c r="D39" s="5"/>
+      <c r="E39" s="5"/>
+      <c r="F39" s="5"/>
+      <c r="G39" s="5"/>
+      <c r="H39" s="5"/>
+      <c r="I39" s="5"/>
+      <c r="J39" s="5"/>
+      <c r="K39" s="5"/>
+      <c r="L39" s="5"/>
+      <c r="M39" s="5"/>
+      <c r="N39" s="5"/>
+      <c r="O39" s="5"/>
+      <c r="P39" s="5"/>
+      <c r="Q39" s="5"/>
+      <c r="R39" s="5"/>
+      <c r="S39" s="5"/>
+      <c r="T39" s="5"/>
+      <c r="U39" s="5"/>
+      <c r="V39" s="5"/>
+      <c r="W39" s="5"/>
+    </row>
+    <row r="40" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A40" s="5"/>
+      <c r="B40" s="5"/>
+      <c r="C40" s="5"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="5"/>
+      <c r="F40" s="5"/>
+      <c r="G40" s="5"/>
+      <c r="H40" s="5"/>
+      <c r="I40" s="5"/>
+      <c r="J40" s="5"/>
+      <c r="K40" s="5"/>
+      <c r="L40" s="5"/>
+      <c r="M40" s="5"/>
+      <c r="N40" s="5"/>
+      <c r="O40" s="5"/>
+      <c r="P40" s="5"/>
+      <c r="Q40" s="5"/>
+      <c r="R40" s="5"/>
+      <c r="S40" s="5"/>
+      <c r="T40" s="5"/>
+      <c r="U40" s="5"/>
+      <c r="V40" s="5"/>
+      <c r="W40" s="5"/>
+    </row>
+    <row r="41" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A41" s="5"/>
+      <c r="B41" s="5"/>
+      <c r="C41" s="5"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="5"/>
+      <c r="I41" s="5"/>
+      <c r="J41" s="5"/>
+      <c r="K41" s="5"/>
+      <c r="L41" s="5"/>
+      <c r="M41" s="5"/>
+      <c r="N41" s="5"/>
+      <c r="O41" s="5"/>
+      <c r="P41" s="5"/>
+      <c r="Q41" s="5"/>
+      <c r="R41" s="5"/>
+      <c r="S41" s="5"/>
+      <c r="T41" s="5"/>
+      <c r="U41" s="5"/>
+      <c r="V41" s="5"/>
+      <c r="W41" s="5"/>
+    </row>
+    <row r="42" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A42" s="5"/>
+      <c r="B42" s="5"/>
+      <c r="C42" s="5"/>
+      <c r="D42" s="5"/>
+      <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
+      <c r="G42" s="5"/>
+      <c r="H42" s="5"/>
+      <c r="I42" s="5"/>
+      <c r="J42" s="5"/>
+      <c r="K42" s="5"/>
+      <c r="L42" s="5"/>
+      <c r="M42" s="5"/>
+      <c r="N42" s="5"/>
+      <c r="O42" s="5"/>
+      <c r="P42" s="5"/>
+      <c r="Q42" s="5"/>
+      <c r="R42" s="5"/>
+      <c r="S42" s="5"/>
+      <c r="T42" s="5"/>
+      <c r="U42" s="5"/>
+      <c r="V42" s="5"/>
+      <c r="W42" s="5"/>
+    </row>
+    <row r="43" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A43" s="5"/>
+      <c r="B43" s="5"/>
+      <c r="C43" s="5"/>
+      <c r="D43" s="5"/>
+      <c r="E43" s="5"/>
+      <c r="F43" s="5"/>
+      <c r="G43" s="5"/>
+      <c r="H43" s="5"/>
+      <c r="I43" s="5"/>
+      <c r="J43" s="5"/>
+      <c r="K43" s="5"/>
+      <c r="L43" s="5"/>
+      <c r="M43" s="5"/>
+      <c r="N43" s="5"/>
+      <c r="O43" s="5"/>
+      <c r="P43" s="5"/>
+      <c r="Q43" s="5"/>
+      <c r="R43" s="5"/>
+      <c r="S43" s="5"/>
+      <c r="T43" s="5"/>
+      <c r="U43" s="5"/>
+      <c r="V43" s="5"/>
+      <c r="W43" s="5"/>
+    </row>
+    <row r="44" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A44" s="5"/>
+      <c r="B44" s="5"/>
+      <c r="C44" s="5"/>
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
+      <c r="F44" s="5"/>
+      <c r="G44" s="5"/>
+      <c r="H44" s="5"/>
+      <c r="I44" s="5"/>
+      <c r="J44" s="5"/>
+      <c r="K44" s="5"/>
+      <c r="L44" s="5"/>
+      <c r="M44" s="5"/>
+      <c r="N44" s="5"/>
+      <c r="O44" s="5"/>
+      <c r="P44" s="5"/>
+      <c r="Q44" s="5"/>
+      <c r="R44" s="5"/>
+      <c r="S44" s="5"/>
+      <c r="T44" s="5"/>
+      <c r="U44" s="5"/>
+      <c r="V44" s="5"/>
+      <c r="W44" s="5"/>
+    </row>
+    <row r="45" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A45" s="5"/>
+      <c r="B45" s="5"/>
+      <c r="C45" s="5"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+      <c r="G45" s="5"/>
+      <c r="H45" s="5"/>
+      <c r="I45" s="5"/>
+      <c r="J45" s="5"/>
+      <c r="K45" s="5"/>
+      <c r="L45" s="5"/>
+      <c r="M45" s="5"/>
+      <c r="N45" s="5"/>
+      <c r="O45" s="5"/>
+      <c r="P45" s="5"/>
+      <c r="Q45" s="5"/>
+      <c r="R45" s="5"/>
+      <c r="S45" s="5"/>
+      <c r="T45" s="5"/>
+      <c r="U45" s="5"/>
+      <c r="V45" s="5"/>
+      <c r="W45" s="5"/>
+    </row>
+    <row r="46" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A46" s="5"/>
+      <c r="B46" s="5"/>
+      <c r="C46" s="5"/>
+      <c r="D46" s="5"/>
+      <c r="E46" s="5"/>
+      <c r="F46" s="5"/>
+      <c r="G46" s="5"/>
+      <c r="H46" s="5"/>
+      <c r="I46" s="5"/>
+      <c r="J46" s="5"/>
+      <c r="K46" s="5"/>
+      <c r="L46" s="5"/>
+      <c r="M46" s="5"/>
+      <c r="N46" s="5"/>
+      <c r="O46" s="5"/>
+      <c r="P46" s="5"/>
+      <c r="Q46" s="5"/>
+      <c r="R46" s="5"/>
+      <c r="S46" s="5"/>
+      <c r="T46" s="5"/>
+      <c r="U46" s="5"/>
+      <c r="V46" s="5"/>
+      <c r="W46" s="5"/>
+    </row>
+    <row r="47" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A47" s="5"/>
+      <c r="B47" s="5"/>
+      <c r="C47" s="5"/>
+      <c r="D47" s="5"/>
+      <c r="E47" s="5"/>
+      <c r="F47" s="5"/>
+      <c r="G47" s="5"/>
+      <c r="H47" s="5"/>
+      <c r="I47" s="5"/>
+      <c r="J47" s="5"/>
+      <c r="K47" s="5"/>
+      <c r="L47" s="5"/>
+      <c r="M47" s="5"/>
+      <c r="N47" s="5"/>
+      <c r="O47" s="5"/>
+      <c r="P47" s="5"/>
+      <c r="Q47" s="5"/>
+      <c r="R47" s="5"/>
+      <c r="S47" s="5"/>
+      <c r="T47" s="5"/>
+      <c r="U47" s="5"/>
+      <c r="V47" s="5"/>
+      <c r="W47" s="5"/>
+    </row>
+    <row r="48" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A48" s="5"/>
+      <c r="B48" s="5"/>
+      <c r="C48" s="5"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="5"/>
+      <c r="F48" s="5"/>
+      <c r="G48" s="5"/>
+      <c r="H48" s="5"/>
+      <c r="I48" s="5"/>
+      <c r="J48" s="5"/>
+      <c r="K48" s="5"/>
+      <c r="L48" s="5"/>
+      <c r="M48" s="5"/>
+      <c r="N48" s="5"/>
+      <c r="O48" s="5"/>
+      <c r="P48" s="5"/>
+      <c r="Q48" s="5"/>
+      <c r="R48" s="5"/>
+      <c r="S48" s="5"/>
+      <c r="T48" s="5"/>
+      <c r="U48" s="5"/>
+      <c r="V48" s="5"/>
+      <c r="W48" s="5"/>
+    </row>
+    <row r="49" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A49" s="5"/>
+      <c r="B49" s="5"/>
+      <c r="C49" s="5"/>
+      <c r="D49" s="5"/>
+      <c r="E49" s="5"/>
+      <c r="F49" s="5"/>
+      <c r="G49" s="5"/>
+      <c r="H49" s="5"/>
+      <c r="I49" s="5"/>
+      <c r="J49" s="5"/>
+      <c r="K49" s="5"/>
+      <c r="L49" s="5"/>
+      <c r="M49" s="5"/>
+      <c r="N49" s="5"/>
+      <c r="O49" s="5"/>
+      <c r="P49" s="5"/>
+      <c r="Q49" s="5"/>
+      <c r="R49" s="5"/>
+      <c r="S49" s="5"/>
+      <c r="T49" s="5"/>
+      <c r="U49" s="5"/>
+      <c r="V49" s="5"/>
+      <c r="W49" s="5"/>
+    </row>
+    <row r="50" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A50" s="5"/>
+      <c r="B50" s="5"/>
+      <c r="C50" s="5"/>
+      <c r="D50" s="5"/>
+      <c r="E50" s="5"/>
+      <c r="F50" s="5"/>
+      <c r="G50" s="5"/>
+      <c r="H50" s="5"/>
+      <c r="I50" s="5"/>
+      <c r="J50" s="5"/>
+      <c r="K50" s="5"/>
+      <c r="L50" s="5"/>
+      <c r="M50" s="5"/>
+      <c r="N50" s="5"/>
+      <c r="O50" s="5"/>
+      <c r="P50" s="5"/>
+      <c r="Q50" s="5"/>
+      <c r="R50" s="5"/>
+      <c r="S50" s="5"/>
+      <c r="T50" s="5"/>
+      <c r="U50" s="5"/>
+      <c r="V50" s="5"/>
+      <c r="W50" s="5"/>
+    </row>
+    <row r="51" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A51" s="5"/>
+      <c r="B51" s="5"/>
+      <c r="C51" s="5"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
+      <c r="G51" s="5"/>
+      <c r="H51" s="5"/>
+      <c r="I51" s="5"/>
+      <c r="J51" s="5"/>
+      <c r="K51" s="5"/>
+      <c r="L51" s="5"/>
+      <c r="M51" s="5"/>
+      <c r="N51" s="5"/>
+      <c r="O51" s="5"/>
+      <c r="P51" s="5"/>
+      <c r="Q51" s="5"/>
+      <c r="R51" s="5"/>
+      <c r="S51" s="5"/>
+      <c r="T51" s="5"/>
+      <c r="U51" s="5"/>
+      <c r="V51" s="5"/>
+      <c r="W51" s="5"/>
+    </row>
+    <row r="52" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A52" s="5"/>
+      <c r="B52" s="5"/>
+      <c r="C52" s="5"/>
+      <c r="D52" s="5"/>
+      <c r="E52" s="5"/>
+      <c r="F52" s="5"/>
+      <c r="G52" s="5"/>
+      <c r="H52" s="5"/>
+      <c r="I52" s="5"/>
+      <c r="J52" s="5"/>
+      <c r="K52" s="5"/>
+      <c r="L52" s="5"/>
+      <c r="M52" s="5"/>
+      <c r="N52" s="5"/>
+      <c r="O52" s="5"/>
+      <c r="P52" s="5"/>
+      <c r="Q52" s="5"/>
+      <c r="R52" s="5"/>
+      <c r="S52" s="5"/>
+      <c r="T52" s="5"/>
+      <c r="U52" s="5"/>
+      <c r="V52" s="5"/>
+      <c r="W52" s="5"/>
+    </row>
+    <row r="53" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A53" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B53" s="5"/>
+      <c r="C53" s="5"/>
+      <c r="D53" s="5"/>
+      <c r="E53" s="5"/>
+      <c r="F53" s="5"/>
+      <c r="G53" s="5"/>
+      <c r="H53" s="5"/>
+      <c r="I53" s="5"/>
+      <c r="J53" s="5"/>
+      <c r="K53" s="5"/>
+      <c r="L53" s="5"/>
+      <c r="M53" s="5"/>
+      <c r="N53" s="5"/>
+      <c r="O53" s="5"/>
+      <c r="P53" s="5"/>
+      <c r="Q53" s="5"/>
+      <c r="R53" s="5"/>
+      <c r="S53" s="5"/>
+      <c r="T53" s="5"/>
+      <c r="U53" s="5"/>
+      <c r="V53" s="5"/>
+      <c r="W53" s="5"/>
+    </row>
+    <row r="54" spans="1:23" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="B54" s="8"/>
+      <c r="C54" s="8"/>
+      <c r="D54" s="8"/>
+      <c r="E54" s="8"/>
+      <c r="F54" s="8"/>
+      <c r="G54" s="8"/>
+      <c r="H54" s="8"/>
+      <c r="I54" s="8"/>
+      <c r="J54" s="8"/>
+      <c r="K54" s="8"/>
+      <c r="L54" s="8"/>
+      <c r="M54" s="8"/>
+      <c r="N54" s="8"/>
+      <c r="O54" s="8"/>
+      <c r="P54" s="8"/>
+      <c r="Q54" s="8"/>
+      <c r="R54" s="8"/>
+      <c r="S54" s="8"/>
+      <c r="T54" s="8"/>
+      <c r="U54" s="8"/>
+      <c r="V54" s="8"/>
+      <c r="W54" s="8"/>
+    </row>
+    <row r="55" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="B55" s="5"/>
+      <c r="C55" s="5"/>
+      <c r="D55" s="5"/>
+      <c r="E55" s="5"/>
+      <c r="F55" s="5"/>
+      <c r="G55" s="5"/>
+      <c r="H55" s="5"/>
+      <c r="I55" s="5"/>
+      <c r="J55" s="5"/>
+      <c r="K55" s="5"/>
+      <c r="L55" s="5"/>
+      <c r="M55" s="5"/>
+      <c r="N55" s="5"/>
+      <c r="O55" s="5"/>
+      <c r="P55" s="5"/>
+      <c r="Q55" s="5"/>
+      <c r="R55" s="5"/>
+      <c r="S55" s="5"/>
+      <c r="T55" s="5"/>
+      <c r="U55" s="5"/>
+      <c r="V55" s="5"/>
+      <c r="W55" s="5"/>
+    </row>
+    <row r="56" spans="1:23" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="B56" s="5"/>
+      <c r="C56" s="5"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
+      <c r="G56" s="5"/>
+      <c r="H56" s="5"/>
+      <c r="I56" s="5"/>
+      <c r="J56" s="5"/>
+      <c r="K56" s="5"/>
+      <c r="L56" s="5"/>
+      <c r="M56" s="5"/>
+      <c r="N56" s="5"/>
+      <c r="O56" s="5"/>
+      <c r="P56" s="5"/>
+      <c r="Q56" s="5"/>
+      <c r="R56" s="5"/>
+      <c r="S56" s="5"/>
+      <c r="T56" s="5"/>
+      <c r="U56" s="5"/>
+      <c r="V56" s="5"/>
+      <c r="W56" s="5"/>
+    </row>
+    <row r="57" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A57" s="5"/>
+      <c r="B57" s="5"/>
+      <c r="C57" s="5"/>
+      <c r="D57" s="5"/>
+      <c r="E57" s="5"/>
+      <c r="F57" s="5"/>
+      <c r="G57" s="5"/>
+      <c r="H57" s="5"/>
+      <c r="I57" s="5"/>
+      <c r="J57" s="5"/>
+      <c r="K57" s="5"/>
+      <c r="L57" s="5"/>
+      <c r="M57" s="5"/>
+      <c r="N57" s="5"/>
+      <c r="O57" s="5"/>
+      <c r="P57" s="5"/>
+      <c r="Q57" s="5"/>
+      <c r="R57" s="5"/>
+      <c r="S57" s="5"/>
+      <c r="T57" s="5"/>
+      <c r="U57" s="5"/>
+      <c r="V57" s="5"/>
+      <c r="W57" s="5"/>
+    </row>
+    <row r="58" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A58" s="5"/>
+      <c r="B58" s="5"/>
+      <c r="C58" s="5"/>
+      <c r="D58" s="5"/>
+      <c r="E58" s="5"/>
+      <c r="F58" s="5"/>
+      <c r="G58" s="5"/>
+      <c r="H58" s="5"/>
+      <c r="I58" s="5"/>
+      <c r="J58" s="5"/>
+      <c r="K58" s="5"/>
+      <c r="L58" s="5"/>
+      <c r="M58" s="5"/>
+      <c r="N58" s="5"/>
+      <c r="O58" s="5"/>
+      <c r="P58" s="5"/>
+      <c r="Q58" s="5"/>
+      <c r="R58" s="5"/>
+      <c r="S58" s="5"/>
+      <c r="T58" s="5"/>
+      <c r="U58" s="5"/>
+      <c r="V58" s="5"/>
+      <c r="W58" s="5"/>
+    </row>
+    <row r="59" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A59" s="5"/>
+      <c r="B59" s="5"/>
+      <c r="C59" s="5"/>
+      <c r="D59" s="5"/>
+      <c r="E59" s="5"/>
+      <c r="F59" s="5"/>
+      <c r="G59" s="5"/>
+      <c r="H59" s="5"/>
+      <c r="I59" s="5"/>
+      <c r="J59" s="5"/>
+      <c r="K59" s="5"/>
+      <c r="L59" s="5"/>
+      <c r="M59" s="5"/>
+      <c r="N59" s="5"/>
+      <c r="O59" s="5"/>
+      <c r="P59" s="5"/>
+      <c r="Q59" s="5"/>
+      <c r="R59" s="5"/>
+      <c r="S59" s="5"/>
+      <c r="T59" s="5"/>
+      <c r="U59" s="5"/>
+      <c r="V59" s="5"/>
+      <c r="W59" s="5"/>
+    </row>
+    <row r="60" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A60" s="5"/>
+      <c r="B60" s="5"/>
+      <c r="C60" s="5"/>
+      <c r="D60" s="5"/>
+      <c r="E60" s="5"/>
+      <c r="F60" s="5"/>
+      <c r="G60" s="5"/>
+      <c r="H60" s="5"/>
+      <c r="I60" s="5"/>
+      <c r="J60" s="5"/>
+      <c r="K60" s="5"/>
+      <c r="L60" s="5"/>
+      <c r="M60" s="5"/>
+      <c r="N60" s="5"/>
+      <c r="O60" s="5"/>
+      <c r="P60" s="5"/>
+      <c r="Q60" s="5"/>
+      <c r="R60" s="5"/>
+      <c r="S60" s="5"/>
+      <c r="T60" s="5"/>
+      <c r="U60" s="5"/>
+      <c r="V60" s="5"/>
+      <c r="W60" s="5"/>
+    </row>
+    <row r="61" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A61" s="5"/>
+      <c r="B61" s="5"/>
+      <c r="C61" s="5"/>
+      <c r="D61" s="5"/>
+      <c r="E61" s="5"/>
+      <c r="F61" s="5"/>
+      <c r="G61" s="5"/>
+      <c r="H61" s="5"/>
+      <c r="I61" s="5"/>
+      <c r="J61" s="5"/>
+      <c r="K61" s="5"/>
+      <c r="L61" s="5"/>
+      <c r="M61" s="5"/>
+      <c r="N61" s="5"/>
+      <c r="O61" s="5"/>
+      <c r="P61" s="5"/>
+      <c r="Q61" s="5"/>
+      <c r="R61" s="5"/>
+      <c r="S61" s="5"/>
+      <c r="T61" s="5"/>
+      <c r="U61" s="5"/>
+      <c r="V61" s="5"/>
+      <c r="W61" s="5"/>
+    </row>
+    <row r="62" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A62" s="5"/>
+      <c r="B62" s="5"/>
+      <c r="C62" s="5"/>
+      <c r="D62" s="5"/>
+      <c r="E62" s="5"/>
+      <c r="F62" s="5"/>
+      <c r="G62" s="5"/>
+      <c r="H62" s="5"/>
+      <c r="I62" s="5"/>
+      <c r="J62" s="5"/>
+      <c r="K62" s="5"/>
+      <c r="L62" s="5"/>
+      <c r="M62" s="5"/>
+      <c r="N62" s="5"/>
+      <c r="O62" s="5"/>
+      <c r="P62" s="5"/>
+      <c r="Q62" s="5"/>
+      <c r="R62" s="5"/>
+      <c r="S62" s="5"/>
+      <c r="T62" s="5"/>
+      <c r="U62" s="5"/>
+      <c r="V62" s="5"/>
+      <c r="W62" s="5"/>
+    </row>
+    <row r="63" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A63" s="5"/>
+      <c r="B63" s="5"/>
+      <c r="C63" s="5"/>
+      <c r="D63" s="5"/>
+      <c r="E63" s="5"/>
+      <c r="F63" s="5"/>
+      <c r="G63" s="5"/>
+      <c r="H63" s="5"/>
+      <c r="I63" s="5"/>
+      <c r="J63" s="5"/>
+      <c r="K63" s="5"/>
+      <c r="L63" s="5"/>
+      <c r="M63" s="5"/>
+      <c r="N63" s="5"/>
+      <c r="O63" s="5"/>
+      <c r="P63" s="5"/>
+      <c r="Q63" s="5"/>
+      <c r="R63" s="5"/>
+      <c r="S63" s="5"/>
+      <c r="T63" s="5"/>
+      <c r="U63" s="5"/>
+      <c r="V63" s="5"/>
+      <c r="W63" s="5"/>
+    </row>
+    <row r="64" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A64" s="5"/>
+      <c r="B64" s="5"/>
+      <c r="C64" s="5"/>
+      <c r="D64" s="5"/>
+      <c r="E64" s="5"/>
+      <c r="F64" s="5"/>
+      <c r="G64" s="5"/>
+      <c r="H64" s="5"/>
+      <c r="I64" s="5"/>
+      <c r="J64" s="5"/>
+      <c r="K64" s="5"/>
+      <c r="L64" s="5"/>
+      <c r="M64" s="5"/>
+      <c r="N64" s="5"/>
+      <c r="O64" s="5"/>
+      <c r="P64" s="5"/>
+      <c r="Q64" s="5"/>
+      <c r="R64" s="5"/>
+      <c r="S64" s="5"/>
+      <c r="T64" s="5"/>
+      <c r="U64" s="5"/>
+      <c r="V64" s="5"/>
+      <c r="W64" s="5"/>
+    </row>
+    <row r="65" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A65" s="5"/>
+      <c r="B65" s="5"/>
+      <c r="C65" s="5"/>
+      <c r="D65" s="5"/>
+      <c r="E65" s="5"/>
+      <c r="F65" s="5"/>
+      <c r="G65" s="5"/>
+      <c r="H65" s="5"/>
+      <c r="I65" s="5"/>
+      <c r="J65" s="5"/>
+      <c r="K65" s="5"/>
+      <c r="L65" s="5"/>
+      <c r="M65" s="5"/>
+      <c r="N65" s="5"/>
+      <c r="O65" s="5"/>
+      <c r="P65" s="5"/>
+      <c r="Q65" s="5"/>
+      <c r="R65" s="5"/>
+      <c r="S65" s="5"/>
+      <c r="T65" s="5"/>
+      <c r="U65" s="5"/>
+      <c r="V65" s="5"/>
+      <c r="W65" s="5"/>
+    </row>
+    <row r="66" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A66" s="5"/>
+      <c r="B66" s="5"/>
+      <c r="C66" s="5"/>
+      <c r="D66" s="5"/>
+      <c r="E66" s="5"/>
+      <c r="F66" s="5"/>
+      <c r="G66" s="5"/>
+      <c r="H66" s="5"/>
+      <c r="I66" s="5"/>
+      <c r="J66" s="5"/>
+      <c r="K66" s="5"/>
+      <c r="L66" s="5"/>
+      <c r="M66" s="5"/>
+      <c r="N66" s="5"/>
+      <c r="O66" s="5"/>
+      <c r="P66" s="5"/>
+      <c r="Q66" s="5"/>
+      <c r="R66" s="5"/>
+      <c r="S66" s="5"/>
+      <c r="T66" s="5"/>
+      <c r="U66" s="5"/>
+      <c r="V66" s="5"/>
+      <c r="W66" s="5"/>
+    </row>
+    <row r="67" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A67" s="5"/>
+      <c r="B67" s="5"/>
+      <c r="C67" s="5"/>
+      <c r="D67" s="5"/>
+      <c r="E67" s="5"/>
+      <c r="F67" s="5"/>
+      <c r="G67" s="5"/>
+      <c r="H67" s="5"/>
+      <c r="I67" s="5"/>
+      <c r="J67" s="5"/>
+      <c r="K67" s="5"/>
+      <c r="L67" s="5"/>
+      <c r="M67" s="5"/>
+      <c r="N67" s="5"/>
+      <c r="O67" s="5"/>
+      <c r="P67" s="5"/>
+      <c r="Q67" s="5"/>
+      <c r="R67" s="5"/>
+      <c r="S67" s="5"/>
+      <c r="T67" s="5"/>
+      <c r="U67" s="5"/>
+      <c r="V67" s="5"/>
+      <c r="W67" s="5"/>
+    </row>
+    <row r="68" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A68" s="5"/>
+      <c r="B68" s="5"/>
+      <c r="C68" s="5"/>
+      <c r="D68" s="5"/>
+      <c r="E68" s="5"/>
+      <c r="F68" s="5"/>
+      <c r="G68" s="5"/>
+      <c r="H68" s="5"/>
+      <c r="I68" s="5"/>
+      <c r="J68" s="5"/>
+      <c r="K68" s="5"/>
+      <c r="L68" s="5"/>
+      <c r="M68" s="5"/>
+      <c r="N68" s="5"/>
+      <c r="O68" s="5"/>
+      <c r="P68" s="5"/>
+      <c r="Q68" s="5"/>
+      <c r="R68" s="5"/>
+      <c r="S68" s="5"/>
+      <c r="T68" s="5"/>
+      <c r="U68" s="5"/>
+      <c r="V68" s="5"/>
+      <c r="W68" s="5"/>
+    </row>
+    <row r="69" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A69" s="5"/>
+      <c r="B69" s="5"/>
+      <c r="C69" s="5"/>
+      <c r="D69" s="5"/>
+      <c r="E69" s="5"/>
+      <c r="F69" s="5"/>
+      <c r="G69" s="5"/>
+      <c r="H69" s="5"/>
+      <c r="I69" s="5"/>
+      <c r="J69" s="5"/>
+      <c r="K69" s="5"/>
+      <c r="L69" s="5"/>
+      <c r="M69" s="5"/>
+      <c r="N69" s="5"/>
+      <c r="O69" s="5"/>
+      <c r="P69" s="5"/>
+      <c r="Q69" s="5"/>
+      <c r="R69" s="5"/>
+      <c r="S69" s="5"/>
+      <c r="T69" s="5"/>
+      <c r="U69" s="5"/>
+      <c r="V69" s="5"/>
+      <c r="W69" s="5"/>
+    </row>
+    <row r="70" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A70" s="5"/>
+      <c r="B70" s="5"/>
+      <c r="C70" s="5"/>
+      <c r="D70" s="5"/>
+      <c r="E70" s="5"/>
+      <c r="F70" s="5"/>
+      <c r="G70" s="5"/>
+      <c r="H70" s="5"/>
+      <c r="I70" s="5"/>
+      <c r="J70" s="5"/>
+      <c r="K70" s="5"/>
+      <c r="L70" s="5"/>
+      <c r="M70" s="5"/>
+      <c r="N70" s="5"/>
+      <c r="O70" s="5"/>
+      <c r="P70" s="5"/>
+      <c r="Q70" s="5"/>
+      <c r="R70" s="5"/>
+      <c r="S70" s="5"/>
+      <c r="T70" s="5"/>
+      <c r="U70" s="5"/>
+      <c r="V70" s="5"/>
+      <c r="W70" s="5"/>
+    </row>
+    <row r="71" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A71" s="5"/>
+      <c r="B71" s="5"/>
+      <c r="C71" s="5"/>
+      <c r="D71" s="5"/>
+      <c r="E71" s="5"/>
+      <c r="F71" s="5"/>
+      <c r="G71" s="5"/>
+      <c r="H71" s="5"/>
+      <c r="I71" s="5"/>
+      <c r="J71" s="5"/>
+      <c r="K71" s="5"/>
+      <c r="L71" s="5"/>
+      <c r="M71" s="5"/>
+      <c r="N71" s="5"/>
+      <c r="O71" s="5"/>
+      <c r="P71" s="5"/>
+      <c r="Q71" s="5"/>
+      <c r="R71" s="5"/>
+      <c r="S71" s="5"/>
+      <c r="T71" s="5"/>
+      <c r="U71" s="5"/>
+      <c r="V71" s="5"/>
+      <c r="W71" s="5"/>
+    </row>
+    <row r="72" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A72" s="5"/>
+      <c r="B72" s="5"/>
+      <c r="C72" s="5"/>
+      <c r="D72" s="5"/>
+      <c r="E72" s="5"/>
+      <c r="F72" s="5"/>
+      <c r="G72" s="5"/>
+      <c r="H72" s="5"/>
+      <c r="I72" s="5"/>
+      <c r="J72" s="5"/>
+      <c r="K72" s="5"/>
+      <c r="L72" s="5"/>
+      <c r="M72" s="5"/>
+      <c r="N72" s="5"/>
+      <c r="O72" s="5"/>
+      <c r="P72" s="5"/>
+      <c r="Q72" s="5"/>
+      <c r="R72" s="5"/>
+      <c r="S72" s="5"/>
+      <c r="T72" s="5"/>
+      <c r="U72" s="5"/>
+      <c r="V72" s="5"/>
+      <c r="W72" s="5"/>
+    </row>
+    <row r="73" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="W73" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:H24"/>
+  <mergeCells count="7">
+    <mergeCell ref="A54:W54"/>
+    <mergeCell ref="A1:W1"/>
+    <mergeCell ref="A7:V7"/>
+    <mergeCell ref="A8:V8"/>
+    <mergeCell ref="A11:V11"/>
+    <mergeCell ref="A17:W17"/>
+    <mergeCell ref="A18:W18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1566,49 +3896,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="2" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
code clean and instructions download pdf
</commit_message>
<xml_diff>
--- a/www/cost-template-empty_Francais.xlsx
+++ b/www/cost-template-empty_Francais.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hthompson\OneDrive - PATH\Documents\github\malaria-budgeting-tool\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF9FDC7F-223B-44C5-8505-A132FABD403E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85319BE1-52AF-47CB-9223-1046FCB0E36B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{E72D83C0-31FE-469B-BB4E-361133B71EB0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{E72D83C0-31FE-469B-BB4E-361133B71EB0}"/>
   </bookViews>
   <sheets>
     <sheet name="instructions" sheetId="3" r:id="rId1"/>
     <sheet name="couts_unitaires_data" sheetId="1" r:id="rId2"/>
     <sheet name="fiches de traitement supplément" sheetId="4" r:id="rId3"/>
-    <sheet name="list-items-ignore" sheetId="2" r:id="rId4"/>
+    <sheet name="liste-options-ignorer" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -1504,9 +1504,6 @@
     <xf numFmtId="0" fontId="14" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="19" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1516,6 +1513,9 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
@@ -2018,31 +2018,31 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:23" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="4"/>
-      <c r="S1" s="4"/>
-      <c r="T1" s="4"/>
-      <c r="U1" s="4"/>
-      <c r="V1" s="4"/>
-      <c r="W1" s="4"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
+      <c r="O1" s="8"/>
+      <c r="P1" s="8"/>
+      <c r="Q1" s="8"/>
+      <c r="R1" s="8"/>
+      <c r="S1" s="8"/>
+      <c r="T1" s="8"/>
+      <c r="U1" s="8"/>
+      <c r="V1" s="8"/>
+      <c r="W1" s="8"/>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
@@ -2053,21 +2053,21 @@
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
-      <c r="O2" s="5"/>
-      <c r="P2" s="5"/>
-      <c r="Q2" s="5"/>
-      <c r="R2" s="5"/>
-      <c r="S2" s="5"/>
-      <c r="T2" s="5"/>
-      <c r="U2" s="5"/>
-      <c r="V2" s="5"/>
-      <c r="W2" s="5"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="4"/>
+      <c r="T2" s="4"/>
+      <c r="U2" s="4"/>
+      <c r="V2" s="4"/>
+      <c r="W2" s="4"/>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
@@ -2078,24 +2078,24 @@
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5"/>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="5"/>
-      <c r="R3" s="5"/>
-      <c r="S3" s="5"/>
-      <c r="T3" s="5"/>
-      <c r="U3" s="5"/>
-      <c r="V3" s="5"/>
-      <c r="W3" s="5"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
+      <c r="S3" s="4"/>
+      <c r="T3" s="4"/>
+      <c r="U3" s="4"/>
+      <c r="V3" s="4"/>
+      <c r="W3" s="4"/>
     </row>
     <row r="4" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="5" t="s">
         <v>98</v>
       </c>
       <c r="B4" s="3"/>
@@ -2105,24 +2105,24 @@
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5"/>
-      <c r="P4" s="5"/>
-      <c r="Q4" s="5"/>
-      <c r="R4" s="5"/>
-      <c r="S4" s="5"/>
-      <c r="T4" s="5"/>
-      <c r="U4" s="5"/>
-      <c r="V4" s="5"/>
-      <c r="W4" s="5"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
+      <c r="R4" s="4"/>
+      <c r="S4" s="4"/>
+      <c r="T4" s="4"/>
+      <c r="U4" s="4"/>
+      <c r="V4" s="4"/>
+      <c r="W4" s="4"/>
     </row>
     <row r="5" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>99</v>
       </c>
       <c r="B5" s="3"/>
@@ -2132,24 +2132,24 @@
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
-      <c r="P5" s="5"/>
-      <c r="Q5" s="5"/>
-      <c r="R5" s="5"/>
-      <c r="S5" s="5"/>
-      <c r="T5" s="5"/>
-      <c r="U5" s="5"/>
-      <c r="V5" s="5"/>
-      <c r="W5" s="5"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
+      <c r="S5" s="4"/>
+      <c r="T5" s="4"/>
+      <c r="U5" s="4"/>
+      <c r="V5" s="4"/>
+      <c r="W5" s="4"/>
     </row>
     <row r="6" spans="1:23" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>100</v>
       </c>
       <c r="B6" s="3"/>
@@ -2159,78 +2159,78 @@
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
-      <c r="O6" s="5"/>
-      <c r="P6" s="5"/>
-      <c r="Q6" s="5"/>
-      <c r="R6" s="5"/>
-      <c r="S6" s="5"/>
-      <c r="T6" s="5"/>
-      <c r="U6" s="5"/>
-      <c r="V6" s="5"/>
-      <c r="W6" s="5"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
+      <c r="L6" s="4"/>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4"/>
+      <c r="Q6" s="4"/>
+      <c r="R6" s="4"/>
+      <c r="S6" s="4"/>
+      <c r="T6" s="4"/>
+      <c r="U6" s="4"/>
+      <c r="V6" s="4"/>
+      <c r="W6" s="4"/>
     </row>
     <row r="7" spans="1:23" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
-      <c r="N7" s="8"/>
-      <c r="O7" s="8"/>
-      <c r="P7" s="8"/>
-      <c r="Q7" s="8"/>
-      <c r="R7" s="8"/>
-      <c r="S7" s="8"/>
-      <c r="T7" s="8"/>
-      <c r="U7" s="8"/>
-      <c r="V7" s="8"/>
-      <c r="W7" s="5"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="7"/>
+      <c r="P7" s="7"/>
+      <c r="Q7" s="7"/>
+      <c r="R7" s="7"/>
+      <c r="S7" s="7"/>
+      <c r="T7" s="7"/>
+      <c r="U7" s="7"/>
+      <c r="V7" s="7"/>
+      <c r="W7" s="4"/>
     </row>
     <row r="8" spans="1:23" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
-      <c r="L8" s="8"/>
-      <c r="M8" s="8"/>
-      <c r="N8" s="8"/>
-      <c r="O8" s="8"/>
-      <c r="P8" s="8"/>
-      <c r="Q8" s="8"/>
-      <c r="R8" s="8"/>
-      <c r="S8" s="8"/>
-      <c r="T8" s="8"/>
-      <c r="U8" s="8"/>
-      <c r="V8" s="8"/>
-      <c r="W8" s="5"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="7"/>
+      <c r="P8" s="7"/>
+      <c r="Q8" s="7"/>
+      <c r="R8" s="7"/>
+      <c r="S8" s="7"/>
+      <c r="T8" s="7"/>
+      <c r="U8" s="7"/>
+      <c r="V8" s="7"/>
+      <c r="W8" s="4"/>
     </row>
     <row r="9" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="5" t="s">
         <v>103</v>
       </c>
       <c r="B9" s="3"/>
@@ -2240,24 +2240,24 @@
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
-      <c r="O9" s="5"/>
-      <c r="P9" s="5"/>
-      <c r="Q9" s="5"/>
-      <c r="R9" s="5"/>
-      <c r="S9" s="5"/>
-      <c r="T9" s="5"/>
-      <c r="U9" s="5"/>
-      <c r="V9" s="5"/>
-      <c r="W9" s="5"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4"/>
+      <c r="Q9" s="4"/>
+      <c r="R9" s="4"/>
+      <c r="S9" s="4"/>
+      <c r="T9" s="4"/>
+      <c r="U9" s="4"/>
+      <c r="V9" s="4"/>
+      <c r="W9" s="4"/>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="6" t="s">
         <v>104</v>
       </c>
       <c r="B10" s="3"/>
@@ -2267,21 +2267,21 @@
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="5"/>
-      <c r="O10" s="5"/>
-      <c r="P10" s="5"/>
-      <c r="Q10" s="5"/>
-      <c r="R10" s="5"/>
-      <c r="S10" s="5"/>
-      <c r="T10" s="5"/>
-      <c r="U10" s="5"/>
-      <c r="V10" s="5"/>
-      <c r="W10" s="5"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="4"/>
+      <c r="Q10" s="4"/>
+      <c r="R10" s="4"/>
+      <c r="S10" s="4"/>
+      <c r="T10" s="4"/>
+      <c r="U10" s="4"/>
+      <c r="V10" s="4"/>
+      <c r="W10" s="4"/>
     </row>
     <row r="11" spans="1:23" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
@@ -2308,10 +2308,10 @@
       <c r="T11" s="9"/>
       <c r="U11" s="9"/>
       <c r="V11" s="9"/>
-      <c r="W11" s="5"/>
+      <c r="W11" s="4"/>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="6" t="s">
         <v>106</v>
       </c>
       <c r="B12" s="3"/>
@@ -2321,24 +2321,24 @@
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
-      <c r="N12" s="5"/>
-      <c r="O12" s="5"/>
-      <c r="P12" s="5"/>
-      <c r="Q12" s="5"/>
-      <c r="R12" s="5"/>
-      <c r="S12" s="5"/>
-      <c r="T12" s="5"/>
-      <c r="U12" s="5"/>
-      <c r="V12" s="5"/>
-      <c r="W12" s="5"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="4"/>
+      <c r="N12" s="4"/>
+      <c r="O12" s="4"/>
+      <c r="P12" s="4"/>
+      <c r="Q12" s="4"/>
+      <c r="R12" s="4"/>
+      <c r="S12" s="4"/>
+      <c r="T12" s="4"/>
+      <c r="U12" s="4"/>
+      <c r="V12" s="4"/>
+      <c r="W12" s="4"/>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="6" t="s">
         <v>107</v>
       </c>
       <c r="B13" s="3"/>
@@ -2348,24 +2348,24 @@
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
-      <c r="N13" s="5"/>
-      <c r="O13" s="5"/>
-      <c r="P13" s="5"/>
-      <c r="Q13" s="5"/>
-      <c r="R13" s="5"/>
-      <c r="S13" s="5"/>
-      <c r="T13" s="5"/>
-      <c r="U13" s="5"/>
-      <c r="V13" s="5"/>
-      <c r="W13" s="5"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+      <c r="L13" s="4"/>
+      <c r="M13" s="4"/>
+      <c r="N13" s="4"/>
+      <c r="O13" s="4"/>
+      <c r="P13" s="4"/>
+      <c r="Q13" s="4"/>
+      <c r="R13" s="4"/>
+      <c r="S13" s="4"/>
+      <c r="T13" s="4"/>
+      <c r="U13" s="4"/>
+      <c r="V13" s="4"/>
+      <c r="W13" s="4"/>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="6" t="s">
         <v>108</v>
       </c>
       <c r="B14" s="3"/>
@@ -2375,24 +2375,24 @@
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
-      <c r="O14" s="5"/>
-      <c r="P14" s="5"/>
-      <c r="Q14" s="5"/>
-      <c r="R14" s="5"/>
-      <c r="S14" s="5"/>
-      <c r="T14" s="5"/>
-      <c r="U14" s="5"/>
-      <c r="V14" s="5"/>
-      <c r="W14" s="5"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+      <c r="L14" s="4"/>
+      <c r="M14" s="4"/>
+      <c r="N14" s="4"/>
+      <c r="O14" s="4"/>
+      <c r="P14" s="4"/>
+      <c r="Q14" s="4"/>
+      <c r="R14" s="4"/>
+      <c r="S14" s="4"/>
+      <c r="T14" s="4"/>
+      <c r="U14" s="4"/>
+      <c r="V14" s="4"/>
+      <c r="W14" s="4"/>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="6" t="s">
         <v>109</v>
       </c>
       <c r="B15" s="3"/>
@@ -2402,24 +2402,24 @@
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
-      <c r="N15" s="5"/>
-      <c r="O15" s="5"/>
-      <c r="P15" s="5"/>
-      <c r="Q15" s="5"/>
-      <c r="R15" s="5"/>
-      <c r="S15" s="5"/>
-      <c r="T15" s="5"/>
-      <c r="U15" s="5"/>
-      <c r="V15" s="5"/>
-      <c r="W15" s="5"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="4"/>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4"/>
+      <c r="O15" s="4"/>
+      <c r="P15" s="4"/>
+      <c r="Q15" s="4"/>
+      <c r="R15" s="4"/>
+      <c r="S15" s="4"/>
+      <c r="T15" s="4"/>
+      <c r="U15" s="4"/>
+      <c r="V15" s="4"/>
+      <c r="W15" s="4"/>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="6" t="s">
         <v>110</v>
       </c>
       <c r="B16" s="3"/>
@@ -2429,21 +2429,21 @@
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
-      <c r="N16" s="5"/>
-      <c r="O16" s="5"/>
-      <c r="P16" s="5"/>
-      <c r="Q16" s="5"/>
-      <c r="R16" s="5"/>
-      <c r="S16" s="5"/>
-      <c r="T16" s="5"/>
-      <c r="U16" s="5"/>
-      <c r="V16" s="5"/>
-      <c r="W16" s="5"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="4"/>
+      <c r="M16" s="4"/>
+      <c r="N16" s="4"/>
+      <c r="O16" s="4"/>
+      <c r="P16" s="4"/>
+      <c r="Q16" s="4"/>
+      <c r="R16" s="4"/>
+      <c r="S16" s="4"/>
+      <c r="T16" s="4"/>
+      <c r="U16" s="4"/>
+      <c r="V16" s="4"/>
+      <c r="W16" s="4"/>
     </row>
     <row r="17" spans="1:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
@@ -2500,7 +2500,7 @@
       <c r="W18" s="9"/>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="6" t="s">
         <v>113</v>
       </c>
       <c r="B19" s="3"/>
@@ -2510,21 +2510,21 @@
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
-      <c r="N19" s="5"/>
-      <c r="O19" s="5"/>
-      <c r="P19" s="5"/>
-      <c r="Q19" s="5"/>
-      <c r="R19" s="5"/>
-      <c r="S19" s="5"/>
-      <c r="T19" s="5"/>
-      <c r="U19" s="5"/>
-      <c r="V19" s="5"/>
-      <c r="W19" s="5"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="4"/>
+      <c r="M19" s="4"/>
+      <c r="N19" s="4"/>
+      <c r="O19" s="4"/>
+      <c r="P19" s="4"/>
+      <c r="Q19" s="4"/>
+      <c r="R19" s="4"/>
+      <c r="S19" s="4"/>
+      <c r="T19" s="4"/>
+      <c r="U19" s="4"/>
+      <c r="V19" s="4"/>
+      <c r="W19" s="4"/>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
@@ -2535,21 +2535,21 @@
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
-      <c r="N20" s="5"/>
-      <c r="O20" s="5"/>
-      <c r="P20" s="5"/>
-      <c r="Q20" s="5"/>
-      <c r="R20" s="5"/>
-      <c r="S20" s="5"/>
-      <c r="T20" s="5"/>
-      <c r="U20" s="5"/>
-      <c r="V20" s="5"/>
-      <c r="W20" s="5"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4"/>
+      <c r="M20" s="4"/>
+      <c r="N20" s="4"/>
+      <c r="O20" s="4"/>
+      <c r="P20" s="4"/>
+      <c r="Q20" s="4"/>
+      <c r="R20" s="4"/>
+      <c r="S20" s="4"/>
+      <c r="T20" s="4"/>
+      <c r="U20" s="4"/>
+      <c r="V20" s="4"/>
+      <c r="W20" s="4"/>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
@@ -2560,21 +2560,21 @@
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
-      <c r="N21" s="5"/>
-      <c r="O21" s="5"/>
-      <c r="P21" s="5"/>
-      <c r="Q21" s="5"/>
-      <c r="R21" s="5"/>
-      <c r="S21" s="5"/>
-      <c r="T21" s="5"/>
-      <c r="U21" s="5"/>
-      <c r="V21" s="5"/>
-      <c r="W21" s="5"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
+      <c r="L21" s="4"/>
+      <c r="M21" s="4"/>
+      <c r="N21" s="4"/>
+      <c r="O21" s="4"/>
+      <c r="P21" s="4"/>
+      <c r="Q21" s="4"/>
+      <c r="R21" s="4"/>
+      <c r="S21" s="4"/>
+      <c r="T21" s="4"/>
+      <c r="U21" s="4"/>
+      <c r="V21" s="4"/>
+      <c r="W21" s="4"/>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
@@ -2585,21 +2585,21 @@
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
-      <c r="I22" s="5"/>
-      <c r="J22" s="5"/>
-      <c r="K22" s="5"/>
-      <c r="L22" s="5"/>
-      <c r="M22" s="5"/>
-      <c r="N22" s="5"/>
-      <c r="O22" s="5"/>
-      <c r="P22" s="5"/>
-      <c r="Q22" s="5"/>
-      <c r="R22" s="5"/>
-      <c r="S22" s="5"/>
-      <c r="T22" s="5"/>
-      <c r="U22" s="5"/>
-      <c r="V22" s="5"/>
-      <c r="W22" s="5"/>
+      <c r="I22" s="4"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
+      <c r="L22" s="4"/>
+      <c r="M22" s="4"/>
+      <c r="N22" s="4"/>
+      <c r="O22" s="4"/>
+      <c r="P22" s="4"/>
+      <c r="Q22" s="4"/>
+      <c r="R22" s="4"/>
+      <c r="S22" s="4"/>
+      <c r="T22" s="4"/>
+      <c r="U22" s="4"/>
+      <c r="V22" s="4"/>
+      <c r="W22" s="4"/>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
@@ -2610,21 +2610,21 @@
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
-      <c r="M23" s="5"/>
-      <c r="N23" s="5"/>
-      <c r="O23" s="5"/>
-      <c r="P23" s="5"/>
-      <c r="Q23" s="5"/>
-      <c r="R23" s="5"/>
-      <c r="S23" s="5"/>
-      <c r="T23" s="5"/>
-      <c r="U23" s="5"/>
-      <c r="V23" s="5"/>
-      <c r="W23" s="5"/>
+      <c r="I23" s="4"/>
+      <c r="J23" s="4"/>
+      <c r="K23" s="4"/>
+      <c r="L23" s="4"/>
+      <c r="M23" s="4"/>
+      <c r="N23" s="4"/>
+      <c r="O23" s="4"/>
+      <c r="P23" s="4"/>
+      <c r="Q23" s="4"/>
+      <c r="R23" s="4"/>
+      <c r="S23" s="4"/>
+      <c r="T23" s="4"/>
+      <c r="U23" s="4"/>
+      <c r="V23" s="4"/>
+      <c r="W23" s="4"/>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
@@ -2635,1232 +2635,1232 @@
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
-      <c r="I24" s="5"/>
-      <c r="J24" s="5"/>
-      <c r="K24" s="5"/>
-      <c r="L24" s="5"/>
-      <c r="M24" s="5"/>
-      <c r="N24" s="5"/>
-      <c r="O24" s="5"/>
-      <c r="P24" s="5"/>
-      <c r="Q24" s="5"/>
-      <c r="R24" s="5"/>
-      <c r="S24" s="5"/>
-      <c r="T24" s="5"/>
-      <c r="U24" s="5"/>
-      <c r="V24" s="5"/>
-      <c r="W24" s="5"/>
+      <c r="I24" s="4"/>
+      <c r="J24" s="4"/>
+      <c r="K24" s="4"/>
+      <c r="L24" s="4"/>
+      <c r="M24" s="4"/>
+      <c r="N24" s="4"/>
+      <c r="O24" s="4"/>
+      <c r="P24" s="4"/>
+      <c r="Q24" s="4"/>
+      <c r="R24" s="4"/>
+      <c r="S24" s="4"/>
+      <c r="T24" s="4"/>
+      <c r="U24" s="4"/>
+      <c r="V24" s="4"/>
+      <c r="W24" s="4"/>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A25" s="5"/>
-      <c r="B25" s="5"/>
-      <c r="C25" s="5"/>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
-      <c r="H25" s="5"/>
-      <c r="I25" s="5"/>
-      <c r="J25" s="5"/>
-      <c r="K25" s="5"/>
-      <c r="L25" s="5"/>
-      <c r="M25" s="5"/>
-      <c r="N25" s="5"/>
-      <c r="O25" s="5"/>
-      <c r="P25" s="5"/>
-      <c r="Q25" s="5"/>
-      <c r="R25" s="5"/>
-      <c r="S25" s="5"/>
-      <c r="T25" s="5"/>
-      <c r="U25" s="5"/>
-      <c r="V25" s="5"/>
-      <c r="W25" s="5"/>
+      <c r="A25" s="4"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
+      <c r="L25" s="4"/>
+      <c r="M25" s="4"/>
+      <c r="N25" s="4"/>
+      <c r="O25" s="4"/>
+      <c r="P25" s="4"/>
+      <c r="Q25" s="4"/>
+      <c r="R25" s="4"/>
+      <c r="S25" s="4"/>
+      <c r="T25" s="4"/>
+      <c r="U25" s="4"/>
+      <c r="V25" s="4"/>
+      <c r="W25" s="4"/>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A26" s="5"/>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
-      <c r="H26" s="5"/>
-      <c r="I26" s="5"/>
-      <c r="J26" s="5"/>
-      <c r="K26" s="5"/>
-      <c r="L26" s="5"/>
-      <c r="M26" s="5"/>
-      <c r="N26" s="5"/>
-      <c r="O26" s="5"/>
-      <c r="P26" s="5"/>
-      <c r="Q26" s="5"/>
-      <c r="R26" s="5"/>
-      <c r="S26" s="5"/>
-      <c r="T26" s="5"/>
-      <c r="U26" s="5"/>
-      <c r="V26" s="5"/>
-      <c r="W26" s="5"/>
+      <c r="A26" s="4"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
+      <c r="K26" s="4"/>
+      <c r="L26" s="4"/>
+      <c r="M26" s="4"/>
+      <c r="N26" s="4"/>
+      <c r="O26" s="4"/>
+      <c r="P26" s="4"/>
+      <c r="Q26" s="4"/>
+      <c r="R26" s="4"/>
+      <c r="S26" s="4"/>
+      <c r="T26" s="4"/>
+      <c r="U26" s="4"/>
+      <c r="V26" s="4"/>
+      <c r="W26" s="4"/>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A27" s="5"/>
-      <c r="B27" s="5"/>
-      <c r="C27" s="5"/>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
-      <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="5"/>
-      <c r="J27" s="5"/>
-      <c r="K27" s="5"/>
-      <c r="L27" s="5"/>
-      <c r="M27" s="5"/>
-      <c r="N27" s="5"/>
-      <c r="O27" s="5"/>
-      <c r="P27" s="5"/>
-      <c r="Q27" s="5"/>
-      <c r="R27" s="5"/>
-      <c r="S27" s="5"/>
-      <c r="T27" s="5"/>
-      <c r="U27" s="5"/>
-      <c r="V27" s="5"/>
-      <c r="W27" s="5"/>
+      <c r="A27" s="4"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="4"/>
+      <c r="J27" s="4"/>
+      <c r="K27" s="4"/>
+      <c r="L27" s="4"/>
+      <c r="M27" s="4"/>
+      <c r="N27" s="4"/>
+      <c r="O27" s="4"/>
+      <c r="P27" s="4"/>
+      <c r="Q27" s="4"/>
+      <c r="R27" s="4"/>
+      <c r="S27" s="4"/>
+      <c r="T27" s="4"/>
+      <c r="U27" s="4"/>
+      <c r="V27" s="4"/>
+      <c r="W27" s="4"/>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A28" s="5"/>
-      <c r="B28" s="5"/>
-      <c r="C28" s="5"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
-      <c r="F28" s="5"/>
-      <c r="G28" s="5"/>
-      <c r="H28" s="5"/>
-      <c r="I28" s="5"/>
-      <c r="J28" s="5"/>
-      <c r="K28" s="5"/>
-      <c r="L28" s="5"/>
-      <c r="M28" s="5"/>
-      <c r="N28" s="5"/>
-      <c r="O28" s="5"/>
-      <c r="P28" s="5"/>
-      <c r="Q28" s="5"/>
-      <c r="R28" s="5"/>
-      <c r="S28" s="5"/>
-      <c r="T28" s="5"/>
-      <c r="U28" s="5"/>
-      <c r="V28" s="5"/>
-      <c r="W28" s="5"/>
+      <c r="A28" s="4"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4"/>
+      <c r="I28" s="4"/>
+      <c r="J28" s="4"/>
+      <c r="K28" s="4"/>
+      <c r="L28" s="4"/>
+      <c r="M28" s="4"/>
+      <c r="N28" s="4"/>
+      <c r="O28" s="4"/>
+      <c r="P28" s="4"/>
+      <c r="Q28" s="4"/>
+      <c r="R28" s="4"/>
+      <c r="S28" s="4"/>
+      <c r="T28" s="4"/>
+      <c r="U28" s="4"/>
+      <c r="V28" s="4"/>
+      <c r="W28" s="4"/>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A29" s="5"/>
-      <c r="B29" s="5"/>
-      <c r="C29" s="5"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5"/>
-      <c r="G29" s="5"/>
-      <c r="H29" s="5"/>
-      <c r="I29" s="5"/>
-      <c r="J29" s="5"/>
-      <c r="K29" s="5"/>
-      <c r="L29" s="5"/>
-      <c r="M29" s="5"/>
-      <c r="N29" s="5"/>
-      <c r="O29" s="5"/>
-      <c r="P29" s="5"/>
-      <c r="Q29" s="5"/>
-      <c r="R29" s="5"/>
-      <c r="S29" s="5"/>
-      <c r="T29" s="5"/>
-      <c r="U29" s="5"/>
-      <c r="V29" s="5"/>
-      <c r="W29" s="5"/>
+      <c r="A29" s="4"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
+      <c r="K29" s="4"/>
+      <c r="L29" s="4"/>
+      <c r="M29" s="4"/>
+      <c r="N29" s="4"/>
+      <c r="O29" s="4"/>
+      <c r="P29" s="4"/>
+      <c r="Q29" s="4"/>
+      <c r="R29" s="4"/>
+      <c r="S29" s="4"/>
+      <c r="T29" s="4"/>
+      <c r="U29" s="4"/>
+      <c r="V29" s="4"/>
+      <c r="W29" s="4"/>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A30" s="5"/>
-      <c r="B30" s="5"/>
-      <c r="C30" s="5"/>
-      <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
-      <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
-      <c r="I30" s="5"/>
-      <c r="J30" s="5"/>
-      <c r="K30" s="5"/>
-      <c r="L30" s="5"/>
-      <c r="M30" s="5"/>
-      <c r="N30" s="5"/>
-      <c r="O30" s="5"/>
-      <c r="P30" s="5"/>
-      <c r="Q30" s="5"/>
-      <c r="R30" s="5"/>
-      <c r="S30" s="5"/>
-      <c r="T30" s="5"/>
-      <c r="U30" s="5"/>
-      <c r="V30" s="5"/>
-      <c r="W30" s="5"/>
+      <c r="A30" s="4"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4"/>
+      <c r="H30" s="4"/>
+      <c r="I30" s="4"/>
+      <c r="J30" s="4"/>
+      <c r="K30" s="4"/>
+      <c r="L30" s="4"/>
+      <c r="M30" s="4"/>
+      <c r="N30" s="4"/>
+      <c r="O30" s="4"/>
+      <c r="P30" s="4"/>
+      <c r="Q30" s="4"/>
+      <c r="R30" s="4"/>
+      <c r="S30" s="4"/>
+      <c r="T30" s="4"/>
+      <c r="U30" s="4"/>
+      <c r="V30" s="4"/>
+      <c r="W30" s="4"/>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A31" s="5"/>
-      <c r="B31" s="5"/>
-      <c r="C31" s="5"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5"/>
-      <c r="G31" s="5"/>
-      <c r="H31" s="5"/>
-      <c r="I31" s="5"/>
-      <c r="J31" s="5"/>
-      <c r="K31" s="5"/>
-      <c r="L31" s="5"/>
-      <c r="M31" s="5"/>
-      <c r="N31" s="5"/>
-      <c r="O31" s="5"/>
-      <c r="P31" s="5"/>
-      <c r="Q31" s="5"/>
-      <c r="R31" s="5"/>
-      <c r="S31" s="5"/>
-      <c r="T31" s="5"/>
-      <c r="U31" s="5"/>
-      <c r="V31" s="5"/>
-      <c r="W31" s="5"/>
+      <c r="A31" s="4"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+      <c r="H31" s="4"/>
+      <c r="I31" s="4"/>
+      <c r="J31" s="4"/>
+      <c r="K31" s="4"/>
+      <c r="L31" s="4"/>
+      <c r="M31" s="4"/>
+      <c r="N31" s="4"/>
+      <c r="O31" s="4"/>
+      <c r="P31" s="4"/>
+      <c r="Q31" s="4"/>
+      <c r="R31" s="4"/>
+      <c r="S31" s="4"/>
+      <c r="T31" s="4"/>
+      <c r="U31" s="4"/>
+      <c r="V31" s="4"/>
+      <c r="W31" s="4"/>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A32" s="5"/>
-      <c r="B32" s="5"/>
-      <c r="C32" s="5"/>
-      <c r="D32" s="5"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5"/>
-      <c r="G32" s="5"/>
-      <c r="H32" s="5"/>
-      <c r="I32" s="5"/>
-      <c r="J32" s="5"/>
-      <c r="K32" s="5"/>
-      <c r="L32" s="5"/>
-      <c r="M32" s="5"/>
-      <c r="N32" s="5"/>
-      <c r="O32" s="5"/>
-      <c r="P32" s="5"/>
-      <c r="Q32" s="5"/>
-      <c r="R32" s="5"/>
-      <c r="S32" s="5"/>
-      <c r="T32" s="5"/>
-      <c r="U32" s="5"/>
-      <c r="V32" s="5"/>
-      <c r="W32" s="5"/>
+      <c r="A32" s="4"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4"/>
+      <c r="H32" s="4"/>
+      <c r="I32" s="4"/>
+      <c r="J32" s="4"/>
+      <c r="K32" s="4"/>
+      <c r="L32" s="4"/>
+      <c r="M32" s="4"/>
+      <c r="N32" s="4"/>
+      <c r="O32" s="4"/>
+      <c r="P32" s="4"/>
+      <c r="Q32" s="4"/>
+      <c r="R32" s="4"/>
+      <c r="S32" s="4"/>
+      <c r="T32" s="4"/>
+      <c r="U32" s="4"/>
+      <c r="V32" s="4"/>
+      <c r="W32" s="4"/>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A33" s="5"/>
-      <c r="B33" s="5"/>
-      <c r="C33" s="5"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
-      <c r="G33" s="5"/>
-      <c r="H33" s="5"/>
-      <c r="I33" s="5"/>
-      <c r="J33" s="5"/>
-      <c r="K33" s="5"/>
-      <c r="L33" s="5"/>
-      <c r="M33" s="5"/>
-      <c r="N33" s="5"/>
-      <c r="O33" s="5"/>
-      <c r="P33" s="5"/>
-      <c r="Q33" s="5"/>
-      <c r="R33" s="5"/>
-      <c r="S33" s="5"/>
-      <c r="T33" s="5"/>
-      <c r="U33" s="5"/>
-      <c r="V33" s="5"/>
-      <c r="W33" s="5"/>
+      <c r="A33" s="4"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
+      <c r="H33" s="4"/>
+      <c r="I33" s="4"/>
+      <c r="J33" s="4"/>
+      <c r="K33" s="4"/>
+      <c r="L33" s="4"/>
+      <c r="M33" s="4"/>
+      <c r="N33" s="4"/>
+      <c r="O33" s="4"/>
+      <c r="P33" s="4"/>
+      <c r="Q33" s="4"/>
+      <c r="R33" s="4"/>
+      <c r="S33" s="4"/>
+      <c r="T33" s="4"/>
+      <c r="U33" s="4"/>
+      <c r="V33" s="4"/>
+      <c r="W33" s="4"/>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A34" s="5"/>
-      <c r="B34" s="5"/>
-      <c r="C34" s="5"/>
-      <c r="D34" s="5"/>
-      <c r="E34" s="5"/>
-      <c r="F34" s="5"/>
-      <c r="G34" s="5"/>
-      <c r="H34" s="5"/>
-      <c r="I34" s="5"/>
-      <c r="J34" s="5"/>
-      <c r="K34" s="5"/>
-      <c r="L34" s="5"/>
-      <c r="M34" s="5"/>
-      <c r="N34" s="5"/>
-      <c r="O34" s="5"/>
-      <c r="P34" s="5"/>
-      <c r="Q34" s="5"/>
-      <c r="R34" s="5"/>
-      <c r="S34" s="5"/>
-      <c r="T34" s="5"/>
-      <c r="U34" s="5"/>
-      <c r="V34" s="5"/>
-      <c r="W34" s="5"/>
+      <c r="A34" s="4"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+      <c r="G34" s="4"/>
+      <c r="H34" s="4"/>
+      <c r="I34" s="4"/>
+      <c r="J34" s="4"/>
+      <c r="K34" s="4"/>
+      <c r="L34" s="4"/>
+      <c r="M34" s="4"/>
+      <c r="N34" s="4"/>
+      <c r="O34" s="4"/>
+      <c r="P34" s="4"/>
+      <c r="Q34" s="4"/>
+      <c r="R34" s="4"/>
+      <c r="S34" s="4"/>
+      <c r="T34" s="4"/>
+      <c r="U34" s="4"/>
+      <c r="V34" s="4"/>
+      <c r="W34" s="4"/>
     </row>
     <row r="35" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A35" s="5"/>
-      <c r="B35" s="5"/>
-      <c r="C35" s="5"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
-      <c r="F35" s="5"/>
-      <c r="G35" s="5"/>
-      <c r="H35" s="5"/>
-      <c r="I35" s="5"/>
-      <c r="J35" s="5"/>
-      <c r="K35" s="5"/>
-      <c r="L35" s="5"/>
-      <c r="M35" s="5"/>
-      <c r="N35" s="5"/>
-      <c r="O35" s="5"/>
-      <c r="P35" s="5"/>
-      <c r="Q35" s="5"/>
-      <c r="R35" s="5"/>
-      <c r="S35" s="5"/>
-      <c r="T35" s="5"/>
-      <c r="U35" s="5"/>
-      <c r="V35" s="5"/>
-      <c r="W35" s="5"/>
+      <c r="A35" s="4"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
+      <c r="G35" s="4"/>
+      <c r="H35" s="4"/>
+      <c r="I35" s="4"/>
+      <c r="J35" s="4"/>
+      <c r="K35" s="4"/>
+      <c r="L35" s="4"/>
+      <c r="M35" s="4"/>
+      <c r="N35" s="4"/>
+      <c r="O35" s="4"/>
+      <c r="P35" s="4"/>
+      <c r="Q35" s="4"/>
+      <c r="R35" s="4"/>
+      <c r="S35" s="4"/>
+      <c r="T35" s="4"/>
+      <c r="U35" s="4"/>
+      <c r="V35" s="4"/>
+      <c r="W35" s="4"/>
     </row>
     <row r="36" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A36" s="5"/>
-      <c r="B36" s="5"/>
-      <c r="C36" s="5"/>
-      <c r="D36" s="5"/>
-      <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
-      <c r="G36" s="5"/>
-      <c r="H36" s="5"/>
-      <c r="I36" s="5"/>
-      <c r="J36" s="5"/>
-      <c r="K36" s="5"/>
-      <c r="L36" s="5"/>
-      <c r="M36" s="5"/>
-      <c r="N36" s="5"/>
-      <c r="O36" s="5"/>
-      <c r="P36" s="5"/>
-      <c r="Q36" s="5"/>
-      <c r="R36" s="5"/>
-      <c r="S36" s="5"/>
-      <c r="T36" s="5"/>
-      <c r="U36" s="5"/>
-      <c r="V36" s="5"/>
-      <c r="W36" s="5"/>
+      <c r="A36" s="4"/>
+      <c r="B36" s="4"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4"/>
+      <c r="G36" s="4"/>
+      <c r="H36" s="4"/>
+      <c r="I36" s="4"/>
+      <c r="J36" s="4"/>
+      <c r="K36" s="4"/>
+      <c r="L36" s="4"/>
+      <c r="M36" s="4"/>
+      <c r="N36" s="4"/>
+      <c r="O36" s="4"/>
+      <c r="P36" s="4"/>
+      <c r="Q36" s="4"/>
+      <c r="R36" s="4"/>
+      <c r="S36" s="4"/>
+      <c r="T36" s="4"/>
+      <c r="U36" s="4"/>
+      <c r="V36" s="4"/>
+      <c r="W36" s="4"/>
     </row>
     <row r="37" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A37" s="5"/>
-      <c r="B37" s="5"/>
-      <c r="C37" s="5"/>
-      <c r="D37" s="5"/>
-      <c r="E37" s="5"/>
-      <c r="F37" s="5"/>
-      <c r="G37" s="5"/>
-      <c r="H37" s="5"/>
-      <c r="I37" s="5"/>
-      <c r="J37" s="5"/>
-      <c r="K37" s="5"/>
-      <c r="L37" s="5"/>
-      <c r="M37" s="5"/>
-      <c r="N37" s="5"/>
-      <c r="O37" s="5"/>
-      <c r="P37" s="5"/>
-      <c r="Q37" s="5"/>
-      <c r="R37" s="5"/>
-      <c r="S37" s="5"/>
-      <c r="T37" s="5"/>
-      <c r="U37" s="5"/>
-      <c r="V37" s="5"/>
-      <c r="W37" s="5"/>
+      <c r="A37" s="4"/>
+      <c r="B37" s="4"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
+      <c r="G37" s="4"/>
+      <c r="H37" s="4"/>
+      <c r="I37" s="4"/>
+      <c r="J37" s="4"/>
+      <c r="K37" s="4"/>
+      <c r="L37" s="4"/>
+      <c r="M37" s="4"/>
+      <c r="N37" s="4"/>
+      <c r="O37" s="4"/>
+      <c r="P37" s="4"/>
+      <c r="Q37" s="4"/>
+      <c r="R37" s="4"/>
+      <c r="S37" s="4"/>
+      <c r="T37" s="4"/>
+      <c r="U37" s="4"/>
+      <c r="V37" s="4"/>
+      <c r="W37" s="4"/>
     </row>
     <row r="38" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A38" s="5"/>
-      <c r="B38" s="5"/>
-      <c r="C38" s="5"/>
-      <c r="D38" s="5"/>
-      <c r="E38" s="5"/>
-      <c r="F38" s="5"/>
-      <c r="G38" s="5"/>
-      <c r="H38" s="5"/>
-      <c r="I38" s="5"/>
-      <c r="J38" s="5"/>
-      <c r="K38" s="5"/>
-      <c r="L38" s="5"/>
-      <c r="M38" s="5"/>
-      <c r="N38" s="5"/>
-      <c r="O38" s="5"/>
-      <c r="P38" s="5"/>
-      <c r="Q38" s="5"/>
-      <c r="R38" s="5"/>
-      <c r="S38" s="5"/>
-      <c r="T38" s="5"/>
-      <c r="U38" s="5"/>
-      <c r="V38" s="5"/>
-      <c r="W38" s="5"/>
+      <c r="A38" s="4"/>
+      <c r="B38" s="4"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="4"/>
+      <c r="F38" s="4"/>
+      <c r="G38" s="4"/>
+      <c r="H38" s="4"/>
+      <c r="I38" s="4"/>
+      <c r="J38" s="4"/>
+      <c r="K38" s="4"/>
+      <c r="L38" s="4"/>
+      <c r="M38" s="4"/>
+      <c r="N38" s="4"/>
+      <c r="O38" s="4"/>
+      <c r="P38" s="4"/>
+      <c r="Q38" s="4"/>
+      <c r="R38" s="4"/>
+      <c r="S38" s="4"/>
+      <c r="T38" s="4"/>
+      <c r="U38" s="4"/>
+      <c r="V38" s="4"/>
+      <c r="W38" s="4"/>
     </row>
     <row r="39" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A39" s="5"/>
-      <c r="B39" s="5"/>
-      <c r="C39" s="5"/>
-      <c r="D39" s="5"/>
-      <c r="E39" s="5"/>
-      <c r="F39" s="5"/>
-      <c r="G39" s="5"/>
-      <c r="H39" s="5"/>
-      <c r="I39" s="5"/>
-      <c r="J39" s="5"/>
-      <c r="K39" s="5"/>
-      <c r="L39" s="5"/>
-      <c r="M39" s="5"/>
-      <c r="N39" s="5"/>
-      <c r="O39" s="5"/>
-      <c r="P39" s="5"/>
-      <c r="Q39" s="5"/>
-      <c r="R39" s="5"/>
-      <c r="S39" s="5"/>
-      <c r="T39" s="5"/>
-      <c r="U39" s="5"/>
-      <c r="V39" s="5"/>
-      <c r="W39" s="5"/>
+      <c r="A39" s="4"/>
+      <c r="B39" s="4"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4"/>
+      <c r="I39" s="4"/>
+      <c r="J39" s="4"/>
+      <c r="K39" s="4"/>
+      <c r="L39" s="4"/>
+      <c r="M39" s="4"/>
+      <c r="N39" s="4"/>
+      <c r="O39" s="4"/>
+      <c r="P39" s="4"/>
+      <c r="Q39" s="4"/>
+      <c r="R39" s="4"/>
+      <c r="S39" s="4"/>
+      <c r="T39" s="4"/>
+      <c r="U39" s="4"/>
+      <c r="V39" s="4"/>
+      <c r="W39" s="4"/>
     </row>
     <row r="40" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A40" s="5"/>
-      <c r="B40" s="5"/>
-      <c r="C40" s="5"/>
-      <c r="D40" s="5"/>
-      <c r="E40" s="5"/>
-      <c r="F40" s="5"/>
-      <c r="G40" s="5"/>
-      <c r="H40" s="5"/>
-      <c r="I40" s="5"/>
-      <c r="J40" s="5"/>
-      <c r="K40" s="5"/>
-      <c r="L40" s="5"/>
-      <c r="M40" s="5"/>
-      <c r="N40" s="5"/>
-      <c r="O40" s="5"/>
-      <c r="P40" s="5"/>
-      <c r="Q40" s="5"/>
-      <c r="R40" s="5"/>
-      <c r="S40" s="5"/>
-      <c r="T40" s="5"/>
-      <c r="U40" s="5"/>
-      <c r="V40" s="5"/>
-      <c r="W40" s="5"/>
+      <c r="A40" s="4"/>
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4"/>
+      <c r="G40" s="4"/>
+      <c r="H40" s="4"/>
+      <c r="I40" s="4"/>
+      <c r="J40" s="4"/>
+      <c r="K40" s="4"/>
+      <c r="L40" s="4"/>
+      <c r="M40" s="4"/>
+      <c r="N40" s="4"/>
+      <c r="O40" s="4"/>
+      <c r="P40" s="4"/>
+      <c r="Q40" s="4"/>
+      <c r="R40" s="4"/>
+      <c r="S40" s="4"/>
+      <c r="T40" s="4"/>
+      <c r="U40" s="4"/>
+      <c r="V40" s="4"/>
+      <c r="W40" s="4"/>
     </row>
     <row r="41" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A41" s="5"/>
-      <c r="B41" s="5"/>
-      <c r="C41" s="5"/>
-      <c r="D41" s="5"/>
-      <c r="E41" s="5"/>
-      <c r="F41" s="5"/>
-      <c r="G41" s="5"/>
-      <c r="H41" s="5"/>
-      <c r="I41" s="5"/>
-      <c r="J41" s="5"/>
-      <c r="K41" s="5"/>
-      <c r="L41" s="5"/>
-      <c r="M41" s="5"/>
-      <c r="N41" s="5"/>
-      <c r="O41" s="5"/>
-      <c r="P41" s="5"/>
-      <c r="Q41" s="5"/>
-      <c r="R41" s="5"/>
-      <c r="S41" s="5"/>
-      <c r="T41" s="5"/>
-      <c r="U41" s="5"/>
-      <c r="V41" s="5"/>
-      <c r="W41" s="5"/>
+      <c r="A41" s="4"/>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="4"/>
+      <c r="H41" s="4"/>
+      <c r="I41" s="4"/>
+      <c r="J41" s="4"/>
+      <c r="K41" s="4"/>
+      <c r="L41" s="4"/>
+      <c r="M41" s="4"/>
+      <c r="N41" s="4"/>
+      <c r="O41" s="4"/>
+      <c r="P41" s="4"/>
+      <c r="Q41" s="4"/>
+      <c r="R41" s="4"/>
+      <c r="S41" s="4"/>
+      <c r="T41" s="4"/>
+      <c r="U41" s="4"/>
+      <c r="V41" s="4"/>
+      <c r="W41" s="4"/>
     </row>
     <row r="42" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A42" s="5"/>
-      <c r="B42" s="5"/>
-      <c r="C42" s="5"/>
-      <c r="D42" s="5"/>
-      <c r="E42" s="5"/>
-      <c r="F42" s="5"/>
-      <c r="G42" s="5"/>
-      <c r="H42" s="5"/>
-      <c r="I42" s="5"/>
-      <c r="J42" s="5"/>
-      <c r="K42" s="5"/>
-      <c r="L42" s="5"/>
-      <c r="M42" s="5"/>
-      <c r="N42" s="5"/>
-      <c r="O42" s="5"/>
-      <c r="P42" s="5"/>
-      <c r="Q42" s="5"/>
-      <c r="R42" s="5"/>
-      <c r="S42" s="5"/>
-      <c r="T42" s="5"/>
-      <c r="U42" s="5"/>
-      <c r="V42" s="5"/>
-      <c r="W42" s="5"/>
+      <c r="A42" s="4"/>
+      <c r="B42" s="4"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="4"/>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
+      <c r="G42" s="4"/>
+      <c r="H42" s="4"/>
+      <c r="I42" s="4"/>
+      <c r="J42" s="4"/>
+      <c r="K42" s="4"/>
+      <c r="L42" s="4"/>
+      <c r="M42" s="4"/>
+      <c r="N42" s="4"/>
+      <c r="O42" s="4"/>
+      <c r="P42" s="4"/>
+      <c r="Q42" s="4"/>
+      <c r="R42" s="4"/>
+      <c r="S42" s="4"/>
+      <c r="T42" s="4"/>
+      <c r="U42" s="4"/>
+      <c r="V42" s="4"/>
+      <c r="W42" s="4"/>
     </row>
     <row r="43" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A43" s="5"/>
-      <c r="B43" s="5"/>
-      <c r="C43" s="5"/>
-      <c r="D43" s="5"/>
-      <c r="E43" s="5"/>
-      <c r="F43" s="5"/>
-      <c r="G43" s="5"/>
-      <c r="H43" s="5"/>
-      <c r="I43" s="5"/>
-      <c r="J43" s="5"/>
-      <c r="K43" s="5"/>
-      <c r="L43" s="5"/>
-      <c r="M43" s="5"/>
-      <c r="N43" s="5"/>
-      <c r="O43" s="5"/>
-      <c r="P43" s="5"/>
-      <c r="Q43" s="5"/>
-      <c r="R43" s="5"/>
-      <c r="S43" s="5"/>
-      <c r="T43" s="5"/>
-      <c r="U43" s="5"/>
-      <c r="V43" s="5"/>
-      <c r="W43" s="5"/>
+      <c r="A43" s="4"/>
+      <c r="B43" s="4"/>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4"/>
+      <c r="F43" s="4"/>
+      <c r="G43" s="4"/>
+      <c r="H43" s="4"/>
+      <c r="I43" s="4"/>
+      <c r="J43" s="4"/>
+      <c r="K43" s="4"/>
+      <c r="L43" s="4"/>
+      <c r="M43" s="4"/>
+      <c r="N43" s="4"/>
+      <c r="O43" s="4"/>
+      <c r="P43" s="4"/>
+      <c r="Q43" s="4"/>
+      <c r="R43" s="4"/>
+      <c r="S43" s="4"/>
+      <c r="T43" s="4"/>
+      <c r="U43" s="4"/>
+      <c r="V43" s="4"/>
+      <c r="W43" s="4"/>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A44" s="5"/>
-      <c r="B44" s="5"/>
-      <c r="C44" s="5"/>
-      <c r="D44" s="5"/>
-      <c r="E44" s="5"/>
-      <c r="F44" s="5"/>
-      <c r="G44" s="5"/>
-      <c r="H44" s="5"/>
-      <c r="I44" s="5"/>
-      <c r="J44" s="5"/>
-      <c r="K44" s="5"/>
-      <c r="L44" s="5"/>
-      <c r="M44" s="5"/>
-      <c r="N44" s="5"/>
-      <c r="O44" s="5"/>
-      <c r="P44" s="5"/>
-      <c r="Q44" s="5"/>
-      <c r="R44" s="5"/>
-      <c r="S44" s="5"/>
-      <c r="T44" s="5"/>
-      <c r="U44" s="5"/>
-      <c r="V44" s="5"/>
-      <c r="W44" s="5"/>
+      <c r="A44" s="4"/>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="E44" s="4"/>
+      <c r="F44" s="4"/>
+      <c r="G44" s="4"/>
+      <c r="H44" s="4"/>
+      <c r="I44" s="4"/>
+      <c r="J44" s="4"/>
+      <c r="K44" s="4"/>
+      <c r="L44" s="4"/>
+      <c r="M44" s="4"/>
+      <c r="N44" s="4"/>
+      <c r="O44" s="4"/>
+      <c r="P44" s="4"/>
+      <c r="Q44" s="4"/>
+      <c r="R44" s="4"/>
+      <c r="S44" s="4"/>
+      <c r="T44" s="4"/>
+      <c r="U44" s="4"/>
+      <c r="V44" s="4"/>
+      <c r="W44" s="4"/>
     </row>
     <row r="45" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A45" s="5"/>
-      <c r="B45" s="5"/>
-      <c r="C45" s="5"/>
-      <c r="D45" s="5"/>
-      <c r="E45" s="5"/>
-      <c r="F45" s="5"/>
-      <c r="G45" s="5"/>
-      <c r="H45" s="5"/>
-      <c r="I45" s="5"/>
-      <c r="J45" s="5"/>
-      <c r="K45" s="5"/>
-      <c r="L45" s="5"/>
-      <c r="M45" s="5"/>
-      <c r="N45" s="5"/>
-      <c r="O45" s="5"/>
-      <c r="P45" s="5"/>
-      <c r="Q45" s="5"/>
-      <c r="R45" s="5"/>
-      <c r="S45" s="5"/>
-      <c r="T45" s="5"/>
-      <c r="U45" s="5"/>
-      <c r="V45" s="5"/>
-      <c r="W45" s="5"/>
+      <c r="A45" s="4"/>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4"/>
+      <c r="G45" s="4"/>
+      <c r="H45" s="4"/>
+      <c r="I45" s="4"/>
+      <c r="J45" s="4"/>
+      <c r="K45" s="4"/>
+      <c r="L45" s="4"/>
+      <c r="M45" s="4"/>
+      <c r="N45" s="4"/>
+      <c r="O45" s="4"/>
+      <c r="P45" s="4"/>
+      <c r="Q45" s="4"/>
+      <c r="R45" s="4"/>
+      <c r="S45" s="4"/>
+      <c r="T45" s="4"/>
+      <c r="U45" s="4"/>
+      <c r="V45" s="4"/>
+      <c r="W45" s="4"/>
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A46" s="5"/>
-      <c r="B46" s="5"/>
-      <c r="C46" s="5"/>
-      <c r="D46" s="5"/>
-      <c r="E46" s="5"/>
-      <c r="F46" s="5"/>
-      <c r="G46" s="5"/>
-      <c r="H46" s="5"/>
-      <c r="I46" s="5"/>
-      <c r="J46" s="5"/>
-      <c r="K46" s="5"/>
-      <c r="L46" s="5"/>
-      <c r="M46" s="5"/>
-      <c r="N46" s="5"/>
-      <c r="O46" s="5"/>
-      <c r="P46" s="5"/>
-      <c r="Q46" s="5"/>
-      <c r="R46" s="5"/>
-      <c r="S46" s="5"/>
-      <c r="T46" s="5"/>
-      <c r="U46" s="5"/>
-      <c r="V46" s="5"/>
-      <c r="W46" s="5"/>
+      <c r="A46" s="4"/>
+      <c r="B46" s="4"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="4"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4"/>
+      <c r="G46" s="4"/>
+      <c r="H46" s="4"/>
+      <c r="I46" s="4"/>
+      <c r="J46" s="4"/>
+      <c r="K46" s="4"/>
+      <c r="L46" s="4"/>
+      <c r="M46" s="4"/>
+      <c r="N46" s="4"/>
+      <c r="O46" s="4"/>
+      <c r="P46" s="4"/>
+      <c r="Q46" s="4"/>
+      <c r="R46" s="4"/>
+      <c r="S46" s="4"/>
+      <c r="T46" s="4"/>
+      <c r="U46" s="4"/>
+      <c r="V46" s="4"/>
+      <c r="W46" s="4"/>
     </row>
     <row r="47" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A47" s="5"/>
-      <c r="B47" s="5"/>
-      <c r="C47" s="5"/>
-      <c r="D47" s="5"/>
-      <c r="E47" s="5"/>
-      <c r="F47" s="5"/>
-      <c r="G47" s="5"/>
-      <c r="H47" s="5"/>
-      <c r="I47" s="5"/>
-      <c r="J47" s="5"/>
-      <c r="K47" s="5"/>
-      <c r="L47" s="5"/>
-      <c r="M47" s="5"/>
-      <c r="N47" s="5"/>
-      <c r="O47" s="5"/>
-      <c r="P47" s="5"/>
-      <c r="Q47" s="5"/>
-      <c r="R47" s="5"/>
-      <c r="S47" s="5"/>
-      <c r="T47" s="5"/>
-      <c r="U47" s="5"/>
-      <c r="V47" s="5"/>
-      <c r="W47" s="5"/>
+      <c r="A47" s="4"/>
+      <c r="B47" s="4"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
+      <c r="F47" s="4"/>
+      <c r="G47" s="4"/>
+      <c r="H47" s="4"/>
+      <c r="I47" s="4"/>
+      <c r="J47" s="4"/>
+      <c r="K47" s="4"/>
+      <c r="L47" s="4"/>
+      <c r="M47" s="4"/>
+      <c r="N47" s="4"/>
+      <c r="O47" s="4"/>
+      <c r="P47" s="4"/>
+      <c r="Q47" s="4"/>
+      <c r="R47" s="4"/>
+      <c r="S47" s="4"/>
+      <c r="T47" s="4"/>
+      <c r="U47" s="4"/>
+      <c r="V47" s="4"/>
+      <c r="W47" s="4"/>
     </row>
     <row r="48" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A48" s="5"/>
-      <c r="B48" s="5"/>
-      <c r="C48" s="5"/>
-      <c r="D48" s="5"/>
-      <c r="E48" s="5"/>
-      <c r="F48" s="5"/>
-      <c r="G48" s="5"/>
-      <c r="H48" s="5"/>
-      <c r="I48" s="5"/>
-      <c r="J48" s="5"/>
-      <c r="K48" s="5"/>
-      <c r="L48" s="5"/>
-      <c r="M48" s="5"/>
-      <c r="N48" s="5"/>
-      <c r="O48" s="5"/>
-      <c r="P48" s="5"/>
-      <c r="Q48" s="5"/>
-      <c r="R48" s="5"/>
-      <c r="S48" s="5"/>
-      <c r="T48" s="5"/>
-      <c r="U48" s="5"/>
-      <c r="V48" s="5"/>
-      <c r="W48" s="5"/>
+      <c r="A48" s="4"/>
+      <c r="B48" s="4"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
+      <c r="G48" s="4"/>
+      <c r="H48" s="4"/>
+      <c r="I48" s="4"/>
+      <c r="J48" s="4"/>
+      <c r="K48" s="4"/>
+      <c r="L48" s="4"/>
+      <c r="M48" s="4"/>
+      <c r="N48" s="4"/>
+      <c r="O48" s="4"/>
+      <c r="P48" s="4"/>
+      <c r="Q48" s="4"/>
+      <c r="R48" s="4"/>
+      <c r="S48" s="4"/>
+      <c r="T48" s="4"/>
+      <c r="U48" s="4"/>
+      <c r="V48" s="4"/>
+      <c r="W48" s="4"/>
     </row>
     <row r="49" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A49" s="5"/>
-      <c r="B49" s="5"/>
-      <c r="C49" s="5"/>
-      <c r="D49" s="5"/>
-      <c r="E49" s="5"/>
-      <c r="F49" s="5"/>
-      <c r="G49" s="5"/>
-      <c r="H49" s="5"/>
-      <c r="I49" s="5"/>
-      <c r="J49" s="5"/>
-      <c r="K49" s="5"/>
-      <c r="L49" s="5"/>
-      <c r="M49" s="5"/>
-      <c r="N49" s="5"/>
-      <c r="O49" s="5"/>
-      <c r="P49" s="5"/>
-      <c r="Q49" s="5"/>
-      <c r="R49" s="5"/>
-      <c r="S49" s="5"/>
-      <c r="T49" s="5"/>
-      <c r="U49" s="5"/>
-      <c r="V49" s="5"/>
-      <c r="W49" s="5"/>
+      <c r="A49" s="4"/>
+      <c r="B49" s="4"/>
+      <c r="C49" s="4"/>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4"/>
+      <c r="F49" s="4"/>
+      <c r="G49" s="4"/>
+      <c r="H49" s="4"/>
+      <c r="I49" s="4"/>
+      <c r="J49" s="4"/>
+      <c r="K49" s="4"/>
+      <c r="L49" s="4"/>
+      <c r="M49" s="4"/>
+      <c r="N49" s="4"/>
+      <c r="O49" s="4"/>
+      <c r="P49" s="4"/>
+      <c r="Q49" s="4"/>
+      <c r="R49" s="4"/>
+      <c r="S49" s="4"/>
+      <c r="T49" s="4"/>
+      <c r="U49" s="4"/>
+      <c r="V49" s="4"/>
+      <c r="W49" s="4"/>
     </row>
     <row r="50" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A50" s="5"/>
-      <c r="B50" s="5"/>
-      <c r="C50" s="5"/>
-      <c r="D50" s="5"/>
-      <c r="E50" s="5"/>
-      <c r="F50" s="5"/>
-      <c r="G50" s="5"/>
-      <c r="H50" s="5"/>
-      <c r="I50" s="5"/>
-      <c r="J50" s="5"/>
-      <c r="K50" s="5"/>
-      <c r="L50" s="5"/>
-      <c r="M50" s="5"/>
-      <c r="N50" s="5"/>
-      <c r="O50" s="5"/>
-      <c r="P50" s="5"/>
-      <c r="Q50" s="5"/>
-      <c r="R50" s="5"/>
-      <c r="S50" s="5"/>
-      <c r="T50" s="5"/>
-      <c r="U50" s="5"/>
-      <c r="V50" s="5"/>
-      <c r="W50" s="5"/>
+      <c r="A50" s="4"/>
+      <c r="B50" s="4"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="4"/>
+      <c r="E50" s="4"/>
+      <c r="F50" s="4"/>
+      <c r="G50" s="4"/>
+      <c r="H50" s="4"/>
+      <c r="I50" s="4"/>
+      <c r="J50" s="4"/>
+      <c r="K50" s="4"/>
+      <c r="L50" s="4"/>
+      <c r="M50" s="4"/>
+      <c r="N50" s="4"/>
+      <c r="O50" s="4"/>
+      <c r="P50" s="4"/>
+      <c r="Q50" s="4"/>
+      <c r="R50" s="4"/>
+      <c r="S50" s="4"/>
+      <c r="T50" s="4"/>
+      <c r="U50" s="4"/>
+      <c r="V50" s="4"/>
+      <c r="W50" s="4"/>
     </row>
     <row r="51" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A51" s="5"/>
-      <c r="B51" s="5"/>
-      <c r="C51" s="5"/>
-      <c r="D51" s="5"/>
-      <c r="E51" s="5"/>
-      <c r="F51" s="5"/>
-      <c r="G51" s="5"/>
-      <c r="H51" s="5"/>
-      <c r="I51" s="5"/>
-      <c r="J51" s="5"/>
-      <c r="K51" s="5"/>
-      <c r="L51" s="5"/>
-      <c r="M51" s="5"/>
-      <c r="N51" s="5"/>
-      <c r="O51" s="5"/>
-      <c r="P51" s="5"/>
-      <c r="Q51" s="5"/>
-      <c r="R51" s="5"/>
-      <c r="S51" s="5"/>
-      <c r="T51" s="5"/>
-      <c r="U51" s="5"/>
-      <c r="V51" s="5"/>
-      <c r="W51" s="5"/>
+      <c r="A51" s="4"/>
+      <c r="B51" s="4"/>
+      <c r="C51" s="4"/>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4"/>
+      <c r="G51" s="4"/>
+      <c r="H51" s="4"/>
+      <c r="I51" s="4"/>
+      <c r="J51" s="4"/>
+      <c r="K51" s="4"/>
+      <c r="L51" s="4"/>
+      <c r="M51" s="4"/>
+      <c r="N51" s="4"/>
+      <c r="O51" s="4"/>
+      <c r="P51" s="4"/>
+      <c r="Q51" s="4"/>
+      <c r="R51" s="4"/>
+      <c r="S51" s="4"/>
+      <c r="T51" s="4"/>
+      <c r="U51" s="4"/>
+      <c r="V51" s="4"/>
+      <c r="W51" s="4"/>
     </row>
     <row r="52" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A52" s="5"/>
-      <c r="B52" s="5"/>
-      <c r="C52" s="5"/>
-      <c r="D52" s="5"/>
-      <c r="E52" s="5"/>
-      <c r="F52" s="5"/>
-      <c r="G52" s="5"/>
-      <c r="H52" s="5"/>
-      <c r="I52" s="5"/>
-      <c r="J52" s="5"/>
-      <c r="K52" s="5"/>
-      <c r="L52" s="5"/>
-      <c r="M52" s="5"/>
-      <c r="N52" s="5"/>
-      <c r="O52" s="5"/>
-      <c r="P52" s="5"/>
-      <c r="Q52" s="5"/>
-      <c r="R52" s="5"/>
-      <c r="S52" s="5"/>
-      <c r="T52" s="5"/>
-      <c r="U52" s="5"/>
-      <c r="V52" s="5"/>
-      <c r="W52" s="5"/>
+      <c r="A52" s="4"/>
+      <c r="B52" s="4"/>
+      <c r="C52" s="4"/>
+      <c r="D52" s="4"/>
+      <c r="E52" s="4"/>
+      <c r="F52" s="4"/>
+      <c r="G52" s="4"/>
+      <c r="H52" s="4"/>
+      <c r="I52" s="4"/>
+      <c r="J52" s="4"/>
+      <c r="K52" s="4"/>
+      <c r="L52" s="4"/>
+      <c r="M52" s="4"/>
+      <c r="N52" s="4"/>
+      <c r="O52" s="4"/>
+      <c r="P52" s="4"/>
+      <c r="Q52" s="4"/>
+      <c r="R52" s="4"/>
+      <c r="S52" s="4"/>
+      <c r="T52" s="4"/>
+      <c r="U52" s="4"/>
+      <c r="V52" s="4"/>
+      <c r="W52" s="4"/>
     </row>
     <row r="53" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A53" s="6" t="s">
+      <c r="A53" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="B53" s="5"/>
-      <c r="C53" s="5"/>
-      <c r="D53" s="5"/>
-      <c r="E53" s="5"/>
-      <c r="F53" s="5"/>
-      <c r="G53" s="5"/>
-      <c r="H53" s="5"/>
-      <c r="I53" s="5"/>
-      <c r="J53" s="5"/>
-      <c r="K53" s="5"/>
-      <c r="L53" s="5"/>
-      <c r="M53" s="5"/>
-      <c r="N53" s="5"/>
-      <c r="O53" s="5"/>
-      <c r="P53" s="5"/>
-      <c r="Q53" s="5"/>
-      <c r="R53" s="5"/>
-      <c r="S53" s="5"/>
-      <c r="T53" s="5"/>
-      <c r="U53" s="5"/>
-      <c r="V53" s="5"/>
-      <c r="W53" s="5"/>
+      <c r="B53" s="4"/>
+      <c r="C53" s="4"/>
+      <c r="D53" s="4"/>
+      <c r="E53" s="4"/>
+      <c r="F53" s="4"/>
+      <c r="G53" s="4"/>
+      <c r="H53" s="4"/>
+      <c r="I53" s="4"/>
+      <c r="J53" s="4"/>
+      <c r="K53" s="4"/>
+      <c r="L53" s="4"/>
+      <c r="M53" s="4"/>
+      <c r="N53" s="4"/>
+      <c r="O53" s="4"/>
+      <c r="P53" s="4"/>
+      <c r="Q53" s="4"/>
+      <c r="R53" s="4"/>
+      <c r="S53" s="4"/>
+      <c r="T53" s="4"/>
+      <c r="U53" s="4"/>
+      <c r="V53" s="4"/>
+      <c r="W53" s="4"/>
     </row>
     <row r="54" spans="1:23" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="8" t="s">
+      <c r="A54" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="B54" s="8"/>
-      <c r="C54" s="8"/>
-      <c r="D54" s="8"/>
-      <c r="E54" s="8"/>
-      <c r="F54" s="8"/>
-      <c r="G54" s="8"/>
-      <c r="H54" s="8"/>
-      <c r="I54" s="8"/>
-      <c r="J54" s="8"/>
-      <c r="K54" s="8"/>
-      <c r="L54" s="8"/>
-      <c r="M54" s="8"/>
-      <c r="N54" s="8"/>
-      <c r="O54" s="8"/>
-      <c r="P54" s="8"/>
-      <c r="Q54" s="8"/>
-      <c r="R54" s="8"/>
-      <c r="S54" s="8"/>
-      <c r="T54" s="8"/>
-      <c r="U54" s="8"/>
-      <c r="V54" s="8"/>
-      <c r="W54" s="8"/>
+      <c r="B54" s="7"/>
+      <c r="C54" s="7"/>
+      <c r="D54" s="7"/>
+      <c r="E54" s="7"/>
+      <c r="F54" s="7"/>
+      <c r="G54" s="7"/>
+      <c r="H54" s="7"/>
+      <c r="I54" s="7"/>
+      <c r="J54" s="7"/>
+      <c r="K54" s="7"/>
+      <c r="L54" s="7"/>
+      <c r="M54" s="7"/>
+      <c r="N54" s="7"/>
+      <c r="O54" s="7"/>
+      <c r="P54" s="7"/>
+      <c r="Q54" s="7"/>
+      <c r="R54" s="7"/>
+      <c r="S54" s="7"/>
+      <c r="T54" s="7"/>
+      <c r="U54" s="7"/>
+      <c r="V54" s="7"/>
+      <c r="W54" s="7"/>
     </row>
     <row r="55" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="6" t="s">
+      <c r="A55" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="B55" s="5"/>
-      <c r="C55" s="5"/>
-      <c r="D55" s="5"/>
-      <c r="E55" s="5"/>
-      <c r="F55" s="5"/>
-      <c r="G55" s="5"/>
-      <c r="H55" s="5"/>
-      <c r="I55" s="5"/>
-      <c r="J55" s="5"/>
-      <c r="K55" s="5"/>
-      <c r="L55" s="5"/>
-      <c r="M55" s="5"/>
-      <c r="N55" s="5"/>
-      <c r="O55" s="5"/>
-      <c r="P55" s="5"/>
-      <c r="Q55" s="5"/>
-      <c r="R55" s="5"/>
-      <c r="S55" s="5"/>
-      <c r="T55" s="5"/>
-      <c r="U55" s="5"/>
-      <c r="V55" s="5"/>
-      <c r="W55" s="5"/>
+      <c r="B55" s="4"/>
+      <c r="C55" s="4"/>
+      <c r="D55" s="4"/>
+      <c r="E55" s="4"/>
+      <c r="F55" s="4"/>
+      <c r="G55" s="4"/>
+      <c r="H55" s="4"/>
+      <c r="I55" s="4"/>
+      <c r="J55" s="4"/>
+      <c r="K55" s="4"/>
+      <c r="L55" s="4"/>
+      <c r="M55" s="4"/>
+      <c r="N55" s="4"/>
+      <c r="O55" s="4"/>
+      <c r="P55" s="4"/>
+      <c r="Q55" s="4"/>
+      <c r="R55" s="4"/>
+      <c r="S55" s="4"/>
+      <c r="T55" s="4"/>
+      <c r="U55" s="4"/>
+      <c r="V55" s="4"/>
+      <c r="W55" s="4"/>
     </row>
     <row r="56" spans="1:23" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="6" t="s">
+      <c r="A56" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="B56" s="5"/>
-      <c r="C56" s="5"/>
-      <c r="D56" s="5"/>
-      <c r="E56" s="5"/>
-      <c r="F56" s="5"/>
-      <c r="G56" s="5"/>
-      <c r="H56" s="5"/>
-      <c r="I56" s="5"/>
-      <c r="J56" s="5"/>
-      <c r="K56" s="5"/>
-      <c r="L56" s="5"/>
-      <c r="M56" s="5"/>
-      <c r="N56" s="5"/>
-      <c r="O56" s="5"/>
-      <c r="P56" s="5"/>
-      <c r="Q56" s="5"/>
-      <c r="R56" s="5"/>
-      <c r="S56" s="5"/>
-      <c r="T56" s="5"/>
-      <c r="U56" s="5"/>
-      <c r="V56" s="5"/>
-      <c r="W56" s="5"/>
+      <c r="B56" s="4"/>
+      <c r="C56" s="4"/>
+      <c r="D56" s="4"/>
+      <c r="E56" s="4"/>
+      <c r="F56" s="4"/>
+      <c r="G56" s="4"/>
+      <c r="H56" s="4"/>
+      <c r="I56" s="4"/>
+      <c r="J56" s="4"/>
+      <c r="K56" s="4"/>
+      <c r="L56" s="4"/>
+      <c r="M56" s="4"/>
+      <c r="N56" s="4"/>
+      <c r="O56" s="4"/>
+      <c r="P56" s="4"/>
+      <c r="Q56" s="4"/>
+      <c r="R56" s="4"/>
+      <c r="S56" s="4"/>
+      <c r="T56" s="4"/>
+      <c r="U56" s="4"/>
+      <c r="V56" s="4"/>
+      <c r="W56" s="4"/>
     </row>
     <row r="57" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A57" s="5"/>
-      <c r="B57" s="5"/>
-      <c r="C57" s="5"/>
-      <c r="D57" s="5"/>
-      <c r="E57" s="5"/>
-      <c r="F57" s="5"/>
-      <c r="G57" s="5"/>
-      <c r="H57" s="5"/>
-      <c r="I57" s="5"/>
-      <c r="J57" s="5"/>
-      <c r="K57" s="5"/>
-      <c r="L57" s="5"/>
-      <c r="M57" s="5"/>
-      <c r="N57" s="5"/>
-      <c r="O57" s="5"/>
-      <c r="P57" s="5"/>
-      <c r="Q57" s="5"/>
-      <c r="R57" s="5"/>
-      <c r="S57" s="5"/>
-      <c r="T57" s="5"/>
-      <c r="U57" s="5"/>
-      <c r="V57" s="5"/>
-      <c r="W57" s="5"/>
+      <c r="A57" s="4"/>
+      <c r="B57" s="4"/>
+      <c r="C57" s="4"/>
+      <c r="D57" s="4"/>
+      <c r="E57" s="4"/>
+      <c r="F57" s="4"/>
+      <c r="G57" s="4"/>
+      <c r="H57" s="4"/>
+      <c r="I57" s="4"/>
+      <c r="J57" s="4"/>
+      <c r="K57" s="4"/>
+      <c r="L57" s="4"/>
+      <c r="M57" s="4"/>
+      <c r="N57" s="4"/>
+      <c r="O57" s="4"/>
+      <c r="P57" s="4"/>
+      <c r="Q57" s="4"/>
+      <c r="R57" s="4"/>
+      <c r="S57" s="4"/>
+      <c r="T57" s="4"/>
+      <c r="U57" s="4"/>
+      <c r="V57" s="4"/>
+      <c r="W57" s="4"/>
     </row>
     <row r="58" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A58" s="5"/>
-      <c r="B58" s="5"/>
-      <c r="C58" s="5"/>
-      <c r="D58" s="5"/>
-      <c r="E58" s="5"/>
-      <c r="F58" s="5"/>
-      <c r="G58" s="5"/>
-      <c r="H58" s="5"/>
-      <c r="I58" s="5"/>
-      <c r="J58" s="5"/>
-      <c r="K58" s="5"/>
-      <c r="L58" s="5"/>
-      <c r="M58" s="5"/>
-      <c r="N58" s="5"/>
-      <c r="O58" s="5"/>
-      <c r="P58" s="5"/>
-      <c r="Q58" s="5"/>
-      <c r="R58" s="5"/>
-      <c r="S58" s="5"/>
-      <c r="T58" s="5"/>
-      <c r="U58" s="5"/>
-      <c r="V58" s="5"/>
-      <c r="W58" s="5"/>
+      <c r="A58" s="4"/>
+      <c r="B58" s="4"/>
+      <c r="C58" s="4"/>
+      <c r="D58" s="4"/>
+      <c r="E58" s="4"/>
+      <c r="F58" s="4"/>
+      <c r="G58" s="4"/>
+      <c r="H58" s="4"/>
+      <c r="I58" s="4"/>
+      <c r="J58" s="4"/>
+      <c r="K58" s="4"/>
+      <c r="L58" s="4"/>
+      <c r="M58" s="4"/>
+      <c r="N58" s="4"/>
+      <c r="O58" s="4"/>
+      <c r="P58" s="4"/>
+      <c r="Q58" s="4"/>
+      <c r="R58" s="4"/>
+      <c r="S58" s="4"/>
+      <c r="T58" s="4"/>
+      <c r="U58" s="4"/>
+      <c r="V58" s="4"/>
+      <c r="W58" s="4"/>
     </row>
     <row r="59" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A59" s="5"/>
-      <c r="B59" s="5"/>
-      <c r="C59" s="5"/>
-      <c r="D59" s="5"/>
-      <c r="E59" s="5"/>
-      <c r="F59" s="5"/>
-      <c r="G59" s="5"/>
-      <c r="H59" s="5"/>
-      <c r="I59" s="5"/>
-      <c r="J59" s="5"/>
-      <c r="K59" s="5"/>
-      <c r="L59" s="5"/>
-      <c r="M59" s="5"/>
-      <c r="N59" s="5"/>
-      <c r="O59" s="5"/>
-      <c r="P59" s="5"/>
-      <c r="Q59" s="5"/>
-      <c r="R59" s="5"/>
-      <c r="S59" s="5"/>
-      <c r="T59" s="5"/>
-      <c r="U59" s="5"/>
-      <c r="V59" s="5"/>
-      <c r="W59" s="5"/>
+      <c r="A59" s="4"/>
+      <c r="B59" s="4"/>
+      <c r="C59" s="4"/>
+      <c r="D59" s="4"/>
+      <c r="E59" s="4"/>
+      <c r="F59" s="4"/>
+      <c r="G59" s="4"/>
+      <c r="H59" s="4"/>
+      <c r="I59" s="4"/>
+      <c r="J59" s="4"/>
+      <c r="K59" s="4"/>
+      <c r="L59" s="4"/>
+      <c r="M59" s="4"/>
+      <c r="N59" s="4"/>
+      <c r="O59" s="4"/>
+      <c r="P59" s="4"/>
+      <c r="Q59" s="4"/>
+      <c r="R59" s="4"/>
+      <c r="S59" s="4"/>
+      <c r="T59" s="4"/>
+      <c r="U59" s="4"/>
+      <c r="V59" s="4"/>
+      <c r="W59" s="4"/>
     </row>
     <row r="60" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A60" s="5"/>
-      <c r="B60" s="5"/>
-      <c r="C60" s="5"/>
-      <c r="D60" s="5"/>
-      <c r="E60" s="5"/>
-      <c r="F60" s="5"/>
-      <c r="G60" s="5"/>
-      <c r="H60" s="5"/>
-      <c r="I60" s="5"/>
-      <c r="J60" s="5"/>
-      <c r="K60" s="5"/>
-      <c r="L60" s="5"/>
-      <c r="M60" s="5"/>
-      <c r="N60" s="5"/>
-      <c r="O60" s="5"/>
-      <c r="P60" s="5"/>
-      <c r="Q60" s="5"/>
-      <c r="R60" s="5"/>
-      <c r="S60" s="5"/>
-      <c r="T60" s="5"/>
-      <c r="U60" s="5"/>
-      <c r="V60" s="5"/>
-      <c r="W60" s="5"/>
+      <c r="A60" s="4"/>
+      <c r="B60" s="4"/>
+      <c r="C60" s="4"/>
+      <c r="D60" s="4"/>
+      <c r="E60" s="4"/>
+      <c r="F60" s="4"/>
+      <c r="G60" s="4"/>
+      <c r="H60" s="4"/>
+      <c r="I60" s="4"/>
+      <c r="J60" s="4"/>
+      <c r="K60" s="4"/>
+      <c r="L60" s="4"/>
+      <c r="M60" s="4"/>
+      <c r="N60" s="4"/>
+      <c r="O60" s="4"/>
+      <c r="P60" s="4"/>
+      <c r="Q60" s="4"/>
+      <c r="R60" s="4"/>
+      <c r="S60" s="4"/>
+      <c r="T60" s="4"/>
+      <c r="U60" s="4"/>
+      <c r="V60" s="4"/>
+      <c r="W60" s="4"/>
     </row>
     <row r="61" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A61" s="5"/>
-      <c r="B61" s="5"/>
-      <c r="C61" s="5"/>
-      <c r="D61" s="5"/>
-      <c r="E61" s="5"/>
-      <c r="F61" s="5"/>
-      <c r="G61" s="5"/>
-      <c r="H61" s="5"/>
-      <c r="I61" s="5"/>
-      <c r="J61" s="5"/>
-      <c r="K61" s="5"/>
-      <c r="L61" s="5"/>
-      <c r="M61" s="5"/>
-      <c r="N61" s="5"/>
-      <c r="O61" s="5"/>
-      <c r="P61" s="5"/>
-      <c r="Q61" s="5"/>
-      <c r="R61" s="5"/>
-      <c r="S61" s="5"/>
-      <c r="T61" s="5"/>
-      <c r="U61" s="5"/>
-      <c r="V61" s="5"/>
-      <c r="W61" s="5"/>
+      <c r="A61" s="4"/>
+      <c r="B61" s="4"/>
+      <c r="C61" s="4"/>
+      <c r="D61" s="4"/>
+      <c r="E61" s="4"/>
+      <c r="F61" s="4"/>
+      <c r="G61" s="4"/>
+      <c r="H61" s="4"/>
+      <c r="I61" s="4"/>
+      <c r="J61" s="4"/>
+      <c r="K61" s="4"/>
+      <c r="L61" s="4"/>
+      <c r="M61" s="4"/>
+      <c r="N61" s="4"/>
+      <c r="O61" s="4"/>
+      <c r="P61" s="4"/>
+      <c r="Q61" s="4"/>
+      <c r="R61" s="4"/>
+      <c r="S61" s="4"/>
+      <c r="T61" s="4"/>
+      <c r="U61" s="4"/>
+      <c r="V61" s="4"/>
+      <c r="W61" s="4"/>
     </row>
     <row r="62" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A62" s="5"/>
-      <c r="B62" s="5"/>
-      <c r="C62" s="5"/>
-      <c r="D62" s="5"/>
-      <c r="E62" s="5"/>
-      <c r="F62" s="5"/>
-      <c r="G62" s="5"/>
-      <c r="H62" s="5"/>
-      <c r="I62" s="5"/>
-      <c r="J62" s="5"/>
-      <c r="K62" s="5"/>
-      <c r="L62" s="5"/>
-      <c r="M62" s="5"/>
-      <c r="N62" s="5"/>
-      <c r="O62" s="5"/>
-      <c r="P62" s="5"/>
-      <c r="Q62" s="5"/>
-      <c r="R62" s="5"/>
-      <c r="S62" s="5"/>
-      <c r="T62" s="5"/>
-      <c r="U62" s="5"/>
-      <c r="V62" s="5"/>
-      <c r="W62" s="5"/>
+      <c r="A62" s="4"/>
+      <c r="B62" s="4"/>
+      <c r="C62" s="4"/>
+      <c r="D62" s="4"/>
+      <c r="E62" s="4"/>
+      <c r="F62" s="4"/>
+      <c r="G62" s="4"/>
+      <c r="H62" s="4"/>
+      <c r="I62" s="4"/>
+      <c r="J62" s="4"/>
+      <c r="K62" s="4"/>
+      <c r="L62" s="4"/>
+      <c r="M62" s="4"/>
+      <c r="N62" s="4"/>
+      <c r="O62" s="4"/>
+      <c r="P62" s="4"/>
+      <c r="Q62" s="4"/>
+      <c r="R62" s="4"/>
+      <c r="S62" s="4"/>
+      <c r="T62" s="4"/>
+      <c r="U62" s="4"/>
+      <c r="V62" s="4"/>
+      <c r="W62" s="4"/>
     </row>
     <row r="63" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A63" s="5"/>
-      <c r="B63" s="5"/>
-      <c r="C63" s="5"/>
-      <c r="D63" s="5"/>
-      <c r="E63" s="5"/>
-      <c r="F63" s="5"/>
-      <c r="G63" s="5"/>
-      <c r="H63" s="5"/>
-      <c r="I63" s="5"/>
-      <c r="J63" s="5"/>
-      <c r="K63" s="5"/>
-      <c r="L63" s="5"/>
-      <c r="M63" s="5"/>
-      <c r="N63" s="5"/>
-      <c r="O63" s="5"/>
-      <c r="P63" s="5"/>
-      <c r="Q63" s="5"/>
-      <c r="R63" s="5"/>
-      <c r="S63" s="5"/>
-      <c r="T63" s="5"/>
-      <c r="U63" s="5"/>
-      <c r="V63" s="5"/>
-      <c r="W63" s="5"/>
+      <c r="A63" s="4"/>
+      <c r="B63" s="4"/>
+      <c r="C63" s="4"/>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4"/>
+      <c r="F63" s="4"/>
+      <c r="G63" s="4"/>
+      <c r="H63" s="4"/>
+      <c r="I63" s="4"/>
+      <c r="J63" s="4"/>
+      <c r="K63" s="4"/>
+      <c r="L63" s="4"/>
+      <c r="M63" s="4"/>
+      <c r="N63" s="4"/>
+      <c r="O63" s="4"/>
+      <c r="P63" s="4"/>
+      <c r="Q63" s="4"/>
+      <c r="R63" s="4"/>
+      <c r="S63" s="4"/>
+      <c r="T63" s="4"/>
+      <c r="U63" s="4"/>
+      <c r="V63" s="4"/>
+      <c r="W63" s="4"/>
     </row>
     <row r="64" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A64" s="5"/>
-      <c r="B64" s="5"/>
-      <c r="C64" s="5"/>
-      <c r="D64" s="5"/>
-      <c r="E64" s="5"/>
-      <c r="F64" s="5"/>
-      <c r="G64" s="5"/>
-      <c r="H64" s="5"/>
-      <c r="I64" s="5"/>
-      <c r="J64" s="5"/>
-      <c r="K64" s="5"/>
-      <c r="L64" s="5"/>
-      <c r="M64" s="5"/>
-      <c r="N64" s="5"/>
-      <c r="O64" s="5"/>
-      <c r="P64" s="5"/>
-      <c r="Q64" s="5"/>
-      <c r="R64" s="5"/>
-      <c r="S64" s="5"/>
-      <c r="T64" s="5"/>
-      <c r="U64" s="5"/>
-      <c r="V64" s="5"/>
-      <c r="W64" s="5"/>
+      <c r="A64" s="4"/>
+      <c r="B64" s="4"/>
+      <c r="C64" s="4"/>
+      <c r="D64" s="4"/>
+      <c r="E64" s="4"/>
+      <c r="F64" s="4"/>
+      <c r="G64" s="4"/>
+      <c r="H64" s="4"/>
+      <c r="I64" s="4"/>
+      <c r="J64" s="4"/>
+      <c r="K64" s="4"/>
+      <c r="L64" s="4"/>
+      <c r="M64" s="4"/>
+      <c r="N64" s="4"/>
+      <c r="O64" s="4"/>
+      <c r="P64" s="4"/>
+      <c r="Q64" s="4"/>
+      <c r="R64" s="4"/>
+      <c r="S64" s="4"/>
+      <c r="T64" s="4"/>
+      <c r="U64" s="4"/>
+      <c r="V64" s="4"/>
+      <c r="W64" s="4"/>
     </row>
     <row r="65" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A65" s="5"/>
-      <c r="B65" s="5"/>
-      <c r="C65" s="5"/>
-      <c r="D65" s="5"/>
-      <c r="E65" s="5"/>
-      <c r="F65" s="5"/>
-      <c r="G65" s="5"/>
-      <c r="H65" s="5"/>
-      <c r="I65" s="5"/>
-      <c r="J65" s="5"/>
-      <c r="K65" s="5"/>
-      <c r="L65" s="5"/>
-      <c r="M65" s="5"/>
-      <c r="N65" s="5"/>
-      <c r="O65" s="5"/>
-      <c r="P65" s="5"/>
-      <c r="Q65" s="5"/>
-      <c r="R65" s="5"/>
-      <c r="S65" s="5"/>
-      <c r="T65" s="5"/>
-      <c r="U65" s="5"/>
-      <c r="V65" s="5"/>
-      <c r="W65" s="5"/>
+      <c r="A65" s="4"/>
+      <c r="B65" s="4"/>
+      <c r="C65" s="4"/>
+      <c r="D65" s="4"/>
+      <c r="E65" s="4"/>
+      <c r="F65" s="4"/>
+      <c r="G65" s="4"/>
+      <c r="H65" s="4"/>
+      <c r="I65" s="4"/>
+      <c r="J65" s="4"/>
+      <c r="K65" s="4"/>
+      <c r="L65" s="4"/>
+      <c r="M65" s="4"/>
+      <c r="N65" s="4"/>
+      <c r="O65" s="4"/>
+      <c r="P65" s="4"/>
+      <c r="Q65" s="4"/>
+      <c r="R65" s="4"/>
+      <c r="S65" s="4"/>
+      <c r="T65" s="4"/>
+      <c r="U65" s="4"/>
+      <c r="V65" s="4"/>
+      <c r="W65" s="4"/>
     </row>
     <row r="66" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A66" s="5"/>
-      <c r="B66" s="5"/>
-      <c r="C66" s="5"/>
-      <c r="D66" s="5"/>
-      <c r="E66" s="5"/>
-      <c r="F66" s="5"/>
-      <c r="G66" s="5"/>
-      <c r="H66" s="5"/>
-      <c r="I66" s="5"/>
-      <c r="J66" s="5"/>
-      <c r="K66" s="5"/>
-      <c r="L66" s="5"/>
-      <c r="M66" s="5"/>
-      <c r="N66" s="5"/>
-      <c r="O66" s="5"/>
-      <c r="P66" s="5"/>
-      <c r="Q66" s="5"/>
-      <c r="R66" s="5"/>
-      <c r="S66" s="5"/>
-      <c r="T66" s="5"/>
-      <c r="U66" s="5"/>
-      <c r="V66" s="5"/>
-      <c r="W66" s="5"/>
+      <c r="A66" s="4"/>
+      <c r="B66" s="4"/>
+      <c r="C66" s="4"/>
+      <c r="D66" s="4"/>
+      <c r="E66" s="4"/>
+      <c r="F66" s="4"/>
+      <c r="G66" s="4"/>
+      <c r="H66" s="4"/>
+      <c r="I66" s="4"/>
+      <c r="J66" s="4"/>
+      <c r="K66" s="4"/>
+      <c r="L66" s="4"/>
+      <c r="M66" s="4"/>
+      <c r="N66" s="4"/>
+      <c r="O66" s="4"/>
+      <c r="P66" s="4"/>
+      <c r="Q66" s="4"/>
+      <c r="R66" s="4"/>
+      <c r="S66" s="4"/>
+      <c r="T66" s="4"/>
+      <c r="U66" s="4"/>
+      <c r="V66" s="4"/>
+      <c r="W66" s="4"/>
     </row>
     <row r="67" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A67" s="5"/>
-      <c r="B67" s="5"/>
-      <c r="C67" s="5"/>
-      <c r="D67" s="5"/>
-      <c r="E67" s="5"/>
-      <c r="F67" s="5"/>
-      <c r="G67" s="5"/>
-      <c r="H67" s="5"/>
-      <c r="I67" s="5"/>
-      <c r="J67" s="5"/>
-      <c r="K67" s="5"/>
-      <c r="L67" s="5"/>
-      <c r="M67" s="5"/>
-      <c r="N67" s="5"/>
-      <c r="O67" s="5"/>
-      <c r="P67" s="5"/>
-      <c r="Q67" s="5"/>
-      <c r="R67" s="5"/>
-      <c r="S67" s="5"/>
-      <c r="T67" s="5"/>
-      <c r="U67" s="5"/>
-      <c r="V67" s="5"/>
-      <c r="W67" s="5"/>
+      <c r="A67" s="4"/>
+      <c r="B67" s="4"/>
+      <c r="C67" s="4"/>
+      <c r="D67" s="4"/>
+      <c r="E67" s="4"/>
+      <c r="F67" s="4"/>
+      <c r="G67" s="4"/>
+      <c r="H67" s="4"/>
+      <c r="I67" s="4"/>
+      <c r="J67" s="4"/>
+      <c r="K67" s="4"/>
+      <c r="L67" s="4"/>
+      <c r="M67" s="4"/>
+      <c r="N67" s="4"/>
+      <c r="O67" s="4"/>
+      <c r="P67" s="4"/>
+      <c r="Q67" s="4"/>
+      <c r="R67" s="4"/>
+      <c r="S67" s="4"/>
+      <c r="T67" s="4"/>
+      <c r="U67" s="4"/>
+      <c r="V67" s="4"/>
+      <c r="W67" s="4"/>
     </row>
     <row r="68" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A68" s="5"/>
-      <c r="B68" s="5"/>
-      <c r="C68" s="5"/>
-      <c r="D68" s="5"/>
-      <c r="E68" s="5"/>
-      <c r="F68" s="5"/>
-      <c r="G68" s="5"/>
-      <c r="H68" s="5"/>
-      <c r="I68" s="5"/>
-      <c r="J68" s="5"/>
-      <c r="K68" s="5"/>
-      <c r="L68" s="5"/>
-      <c r="M68" s="5"/>
-      <c r="N68" s="5"/>
-      <c r="O68" s="5"/>
-      <c r="P68" s="5"/>
-      <c r="Q68" s="5"/>
-      <c r="R68" s="5"/>
-      <c r="S68" s="5"/>
-      <c r="T68" s="5"/>
-      <c r="U68" s="5"/>
-      <c r="V68" s="5"/>
-      <c r="W68" s="5"/>
+      <c r="A68" s="4"/>
+      <c r="B68" s="4"/>
+      <c r="C68" s="4"/>
+      <c r="D68" s="4"/>
+      <c r="E68" s="4"/>
+      <c r="F68" s="4"/>
+      <c r="G68" s="4"/>
+      <c r="H68" s="4"/>
+      <c r="I68" s="4"/>
+      <c r="J68" s="4"/>
+      <c r="K68" s="4"/>
+      <c r="L68" s="4"/>
+      <c r="M68" s="4"/>
+      <c r="N68" s="4"/>
+      <c r="O68" s="4"/>
+      <c r="P68" s="4"/>
+      <c r="Q68" s="4"/>
+      <c r="R68" s="4"/>
+      <c r="S68" s="4"/>
+      <c r="T68" s="4"/>
+      <c r="U68" s="4"/>
+      <c r="V68" s="4"/>
+      <c r="W68" s="4"/>
     </row>
     <row r="69" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A69" s="5"/>
-      <c r="B69" s="5"/>
-      <c r="C69" s="5"/>
-      <c r="D69" s="5"/>
-      <c r="E69" s="5"/>
-      <c r="F69" s="5"/>
-      <c r="G69" s="5"/>
-      <c r="H69" s="5"/>
-      <c r="I69" s="5"/>
-      <c r="J69" s="5"/>
-      <c r="K69" s="5"/>
-      <c r="L69" s="5"/>
-      <c r="M69" s="5"/>
-      <c r="N69" s="5"/>
-      <c r="O69" s="5"/>
-      <c r="P69" s="5"/>
-      <c r="Q69" s="5"/>
-      <c r="R69" s="5"/>
-      <c r="S69" s="5"/>
-      <c r="T69" s="5"/>
-      <c r="U69" s="5"/>
-      <c r="V69" s="5"/>
-      <c r="W69" s="5"/>
+      <c r="A69" s="4"/>
+      <c r="B69" s="4"/>
+      <c r="C69" s="4"/>
+      <c r="D69" s="4"/>
+      <c r="E69" s="4"/>
+      <c r="F69" s="4"/>
+      <c r="G69" s="4"/>
+      <c r="H69" s="4"/>
+      <c r="I69" s="4"/>
+      <c r="J69" s="4"/>
+      <c r="K69" s="4"/>
+      <c r="L69" s="4"/>
+      <c r="M69" s="4"/>
+      <c r="N69" s="4"/>
+      <c r="O69" s="4"/>
+      <c r="P69" s="4"/>
+      <c r="Q69" s="4"/>
+      <c r="R69" s="4"/>
+      <c r="S69" s="4"/>
+      <c r="T69" s="4"/>
+      <c r="U69" s="4"/>
+      <c r="V69" s="4"/>
+      <c r="W69" s="4"/>
     </row>
     <row r="70" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A70" s="5"/>
-      <c r="B70" s="5"/>
-      <c r="C70" s="5"/>
-      <c r="D70" s="5"/>
-      <c r="E70" s="5"/>
-      <c r="F70" s="5"/>
-      <c r="G70" s="5"/>
-      <c r="H70" s="5"/>
-      <c r="I70" s="5"/>
-      <c r="J70" s="5"/>
-      <c r="K70" s="5"/>
-      <c r="L70" s="5"/>
-      <c r="M70" s="5"/>
-      <c r="N70" s="5"/>
-      <c r="O70" s="5"/>
-      <c r="P70" s="5"/>
-      <c r="Q70" s="5"/>
-      <c r="R70" s="5"/>
-      <c r="S70" s="5"/>
-      <c r="T70" s="5"/>
-      <c r="U70" s="5"/>
-      <c r="V70" s="5"/>
-      <c r="W70" s="5"/>
+      <c r="A70" s="4"/>
+      <c r="B70" s="4"/>
+      <c r="C70" s="4"/>
+      <c r="D70" s="4"/>
+      <c r="E70" s="4"/>
+      <c r="F70" s="4"/>
+      <c r="G70" s="4"/>
+      <c r="H70" s="4"/>
+      <c r="I70" s="4"/>
+      <c r="J70" s="4"/>
+      <c r="K70" s="4"/>
+      <c r="L70" s="4"/>
+      <c r="M70" s="4"/>
+      <c r="N70" s="4"/>
+      <c r="O70" s="4"/>
+      <c r="P70" s="4"/>
+      <c r="Q70" s="4"/>
+      <c r="R70" s="4"/>
+      <c r="S70" s="4"/>
+      <c r="T70" s="4"/>
+      <c r="U70" s="4"/>
+      <c r="V70" s="4"/>
+      <c r="W70" s="4"/>
     </row>
     <row r="71" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A71" s="5"/>
-      <c r="B71" s="5"/>
-      <c r="C71" s="5"/>
-      <c r="D71" s="5"/>
-      <c r="E71" s="5"/>
-      <c r="F71" s="5"/>
-      <c r="G71" s="5"/>
-      <c r="H71" s="5"/>
-      <c r="I71" s="5"/>
-      <c r="J71" s="5"/>
-      <c r="K71" s="5"/>
-      <c r="L71" s="5"/>
-      <c r="M71" s="5"/>
-      <c r="N71" s="5"/>
-      <c r="O71" s="5"/>
-      <c r="P71" s="5"/>
-      <c r="Q71" s="5"/>
-      <c r="R71" s="5"/>
-      <c r="S71" s="5"/>
-      <c r="T71" s="5"/>
-      <c r="U71" s="5"/>
-      <c r="V71" s="5"/>
-      <c r="W71" s="5"/>
+      <c r="A71" s="4"/>
+      <c r="B71" s="4"/>
+      <c r="C71" s="4"/>
+      <c r="D71" s="4"/>
+      <c r="E71" s="4"/>
+      <c r="F71" s="4"/>
+      <c r="G71" s="4"/>
+      <c r="H71" s="4"/>
+      <c r="I71" s="4"/>
+      <c r="J71" s="4"/>
+      <c r="K71" s="4"/>
+      <c r="L71" s="4"/>
+      <c r="M71" s="4"/>
+      <c r="N71" s="4"/>
+      <c r="O71" s="4"/>
+      <c r="P71" s="4"/>
+      <c r="Q71" s="4"/>
+      <c r="R71" s="4"/>
+      <c r="S71" s="4"/>
+      <c r="T71" s="4"/>
+      <c r="U71" s="4"/>
+      <c r="V71" s="4"/>
+      <c r="W71" s="4"/>
     </row>
     <row r="72" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A72" s="5"/>
-      <c r="B72" s="5"/>
-      <c r="C72" s="5"/>
-      <c r="D72" s="5"/>
-      <c r="E72" s="5"/>
-      <c r="F72" s="5"/>
-      <c r="G72" s="5"/>
-      <c r="H72" s="5"/>
-      <c r="I72" s="5"/>
-      <c r="J72" s="5"/>
-      <c r="K72" s="5"/>
-      <c r="L72" s="5"/>
-      <c r="M72" s="5"/>
-      <c r="N72" s="5"/>
-      <c r="O72" s="5"/>
-      <c r="P72" s="5"/>
-      <c r="Q72" s="5"/>
-      <c r="R72" s="5"/>
-      <c r="S72" s="5"/>
-      <c r="T72" s="5"/>
-      <c r="U72" s="5"/>
-      <c r="V72" s="5"/>
-      <c r="W72" s="5"/>
+      <c r="A72" s="4"/>
+      <c r="B72" s="4"/>
+      <c r="C72" s="4"/>
+      <c r="D72" s="4"/>
+      <c r="E72" s="4"/>
+      <c r="F72" s="4"/>
+      <c r="G72" s="4"/>
+      <c r="H72" s="4"/>
+      <c r="I72" s="4"/>
+      <c r="J72" s="4"/>
+      <c r="K72" s="4"/>
+      <c r="L72" s="4"/>
+      <c r="M72" s="4"/>
+      <c r="N72" s="4"/>
+      <c r="O72" s="4"/>
+      <c r="P72" s="4"/>
+      <c r="Q72" s="4"/>
+      <c r="R72" s="4"/>
+      <c r="S72" s="4"/>
+      <c r="T72" s="4"/>
+      <c r="U72" s="4"/>
+      <c r="V72" s="4"/>
+      <c r="W72" s="4"/>
     </row>
     <row r="73" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="W73" s="5"/>
+      <c r="W73" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -4349,19 +4349,19 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2B23E79F-74DE-47A3-AA72-02125CE1366C}">
           <x14:formula1>
-            <xm:f>'list-items-ignore'!$B$1:$B$10</xm:f>
+            <xm:f>'liste-options-ignorer'!$B$1:$B$10</xm:f>
           </x14:formula1>
           <xm:sqref>A2:A1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E5E138DD-4BA1-445F-A665-4841EF8F02BE}">
           <x14:formula1>
-            <xm:f>'list-items-ignore'!$D:$D</xm:f>
+            <xm:f>'liste-options-ignorer'!$D:$D</xm:f>
           </x14:formula1>
           <xm:sqref>B2:B1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{613C0C3E-E487-435C-8D59-412773A42907}">
           <x14:formula1>
-            <xm:f>'list-items-ignore'!$G:$G</xm:f>
+            <xm:f>'liste-options-ignorer'!$G:$G</xm:f>
           </x14:formula1>
           <xm:sqref>F30:F1048576</xm:sqref>
         </x14:dataValidation>

</xml_diff>